<commit_message>
chore: bazar_watcher data update 2026-09-13
</commit_message>
<xml_diff>
--- a/data/bazar_watcher/listings.xlsx
+++ b/data/bazar_watcher/listings.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M616"/>
+  <dimension ref="A1:M621"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -33873,11 +33873,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-dls-26-7734/</t>
         </is>
       </c>
-      <c r="F613" t="n">
-        <v>1700</v>
-      </c>
-      <c r="G613" t="n">
-        <v>2023</v>
+      <c r="F613" t="inlineStr">
+        <is>
+          <t>1700.0</t>
+        </is>
+      </c>
+      <c r="G613" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
       </c>
       <c r="H613" t="inlineStr">
         <is>
@@ -33929,8 +33933,10 @@
         </is>
       </c>
       <c r="F614" t="inlineStr"/>
-      <c r="G614" t="n">
-        <v>2020</v>
+      <c r="G614" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
       </c>
       <c r="H614" t="inlineStr">
         <is>
@@ -33982,8 +33988,10 @@
         </is>
       </c>
       <c r="F615" t="inlineStr"/>
-      <c r="G615" t="n">
-        <v>2019</v>
+      <c r="G615" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
       </c>
       <c r="H615" t="inlineStr">
         <is>
@@ -34035,8 +34043,10 @@
         </is>
       </c>
       <c r="F616" t="inlineStr"/>
-      <c r="G616" t="n">
-        <v>2005</v>
+      <c r="G616" t="inlineStr">
+        <is>
+          <t>2005</t>
+        </is>
       </c>
       <c r="H616" t="inlineStr">
         <is>
@@ -34058,6 +34068,277 @@
       <c r="M616" t="inlineStr">
         <is>
           <t>2026-09-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="617">
+      <c r="A617" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B617" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C617" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D617" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Ozone Buzz z4 S 65-85kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B Ozon</t>
+        </is>
+      </c>
+      <c r="E617" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/ozone-buzz-z4-s-65-85kg-concertinas-no-sivs-no-flying-on-7753/</t>
+        </is>
+      </c>
+      <c r="F617" t="inlineStr"/>
+      <c r="G617" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H617" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I617" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J617" t="inlineStr"/>
+      <c r="K617" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L617" t="inlineStr"/>
+      <c r="M617" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="618">
+      <c r="A618" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B618" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C618" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D618" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Gradient Golden 4 26 85-100kg TK čerstvá TK platná S listovacím obalem Křídlo EN B Gradient Golden 4 26 85-1</t>
+        </is>
+      </c>
+      <c r="E618" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/gradient-golden-4-26-85-100kg-tc-fresh-tc-valid-with-lis-7751/</t>
+        </is>
+      </c>
+      <c r="F618" t="n">
+        <v>620</v>
+      </c>
+      <c r="G618" t="n">
+        <v>2016</v>
+      </c>
+      <c r="H618" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I618" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="J618" t="inlineStr"/>
+      <c r="K618" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L618" t="inlineStr"/>
+      <c r="M618" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="619">
+      <c r="A619" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B619" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C619" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D619" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Advance Epsilon DLS 26 Křídlo EN B Advance Epsilon DLS 26 41 225,11 CZK (1 700,00 EUR) EN B Velikost: 26 Opo</t>
+        </is>
+      </c>
+      <c r="E619" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-dls-26-7734/</t>
+        </is>
+      </c>
+      <c r="F619" t="n">
+        <v>1700</v>
+      </c>
+      <c r="G619" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H619" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I619" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="J619" t="inlineStr"/>
+      <c r="K619" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L619" t="inlineStr"/>
+      <c r="M619" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="620">
+      <c r="A620" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B620" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C620" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D620" t="inlineStr">
+        <is>
+          <t>Křídlo EN B MAC Eden 7 26 80-105kg TK čerstvá TK platná Křídlo EN B MAC Eden 7 26 80-105kg TK čerstvá TK platná 18 000,0</t>
+        </is>
+      </c>
+      <c r="E620" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/mac-eden-7-26-80-105kg-tc-fresh-tc-valid-7593/</t>
+        </is>
+      </c>
+      <c r="F620" t="inlineStr"/>
+      <c r="G620" t="n">
+        <v>2022</v>
+      </c>
+      <c r="H620" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I620" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="J620" t="inlineStr"/>
+      <c r="K620" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L620" t="inlineStr"/>
+      <c r="M620" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="621">
+      <c r="A621" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B621" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C621" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D621" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Drift carancho S 69-90kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN A Drift caranch</t>
+        </is>
+      </c>
+      <c r="E621" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/drift-carancho-s-69-90kg-no-sivs-no-flying-on-the-sand-n-7752/</t>
+        </is>
+      </c>
+      <c r="F621" t="n">
+        <v>1800</v>
+      </c>
+      <c r="G621" t="n">
+        <v>2024</v>
+      </c>
+      <c r="H621" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I621" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J621" t="inlineStr"/>
+      <c r="K621" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L621" t="inlineStr"/>
+      <c r="M621" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
         </is>
       </c>
     </row>
@@ -34072,7 +34353,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M30"/>
+  <dimension ref="A1:M35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -35526,11 +35807,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-dls-26-7734/</t>
         </is>
       </c>
-      <c r="F27" t="n">
-        <v>1700</v>
-      </c>
-      <c r="G27" t="n">
-        <v>2023</v>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>1700.0</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
@@ -35582,8 +35867,10 @@
         </is>
       </c>
       <c r="F28" t="inlineStr"/>
-      <c r="G28" t="n">
-        <v>2020</v>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
@@ -35635,8 +35922,10 @@
         </is>
       </c>
       <c r="F29" t="inlineStr"/>
-      <c r="G29" t="n">
-        <v>2019</v>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
@@ -35688,8 +35977,10 @@
         </is>
       </c>
       <c r="F30" t="inlineStr"/>
-      <c r="G30" t="n">
-        <v>2005</v>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>2005</t>
+        </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
@@ -35711,6 +36002,277 @@
       <c r="M30" t="inlineStr">
         <is>
           <t>2026-09-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Ozone Buzz z4 S 65-85kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B Ozon</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/ozone-buzz-z4-s-65-85kg-concertinas-no-sivs-no-flying-on-7753/</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr"/>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Gradient Golden 4 26 85-100kg TK čerstvá TK platná S listovacím obalem Křídlo EN B Gradient Golden 4 26 85-1</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/gradient-golden-4-26-85-100kg-tc-fresh-tc-valid-with-lis-7751/</t>
+        </is>
+      </c>
+      <c r="F32" t="n">
+        <v>620</v>
+      </c>
+      <c r="G32" t="n">
+        <v>2016</v>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr"/>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr"/>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Advance Epsilon DLS 26 Křídlo EN B Advance Epsilon DLS 26 41 225,11 CZK (1 700,00 EUR) EN B Velikost: 26 Opo</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-dls-26-7734/</t>
+        </is>
+      </c>
+      <c r="F33" t="n">
+        <v>1700</v>
+      </c>
+      <c r="G33" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr"/>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr"/>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Křídlo EN B MAC Eden 7 26 80-105kg TK čerstvá TK platná Křídlo EN B MAC Eden 7 26 80-105kg TK čerstvá TK platná 18 000,0</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/mac-eden-7-26-80-105kg-tc-fresh-tc-valid-7593/</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="n">
+        <v>2022</v>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr"/>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr"/>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Drift carancho S 69-90kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN A Drift caranch</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/drift-carancho-s-69-90kg-no-sivs-no-flying-on-the-sand-n-7752/</t>
+        </is>
+      </c>
+      <c r="F35" t="n">
+        <v>1800</v>
+      </c>
+      <c r="G35" t="n">
+        <v>2024</v>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr"/>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr"/>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
         </is>
       </c>
     </row>
@@ -35725,7 +36287,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M5"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -35828,19 +36390,17 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN B Advance Epsilon DLS 26 Křídlo EN B Advance Epsilon DLS 26 41 242,12 CZK (1 700,00 EUR) EN B Velikost: 26 Opo</t>
+          <t>Křídlo EN B Ozone Buzz z4 S 65-85kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B Ozon</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-dls-26-7734/</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>1700</v>
-      </c>
+          <t>https://paragliding-bazar.cz/cs/offering/ozone-buzz-z4-s-65-85kg-concertinas-no-sivs-no-flying-on-7753/</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
       <c r="G2" t="n">
-        <v>2023</v>
+        <v>2015</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -35849,31 +36409,31 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>S</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Létané (100-200h)</t>
+          <t>Jako nové (0-50h)</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_a</t>
+          <t>paragliding_bazar_cz_b</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN A</t>
+          <t>Paragliding Bazar CZ – EN B</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -35883,50 +36443,52 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Křídlo EN A Gradient Golden 4 24 75-100kg Listovaný Žádné SIV Nelétáno na písku Nekoupáno TK čerstvá Křídlo EN A Gradien</t>
+          <t>Křídlo EN B Gradient Golden 4 26 85-100kg TK čerstvá TK platná S listovacím obalem Křídlo EN B Gradient Golden 4 26 85-1</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/gradient-golden-4-24-75-100kg-concertinas-no-sivs-no-fly-7749/</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
+          <t>https://paragliding-bazar.cz/cs/offering/gradient-golden-4-26-85-100kg-tc-fresh-tc-valid-with-lis-7751/</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>620</v>
+      </c>
       <c r="G3" t="n">
-        <v>2020</v>
+        <v>2016</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>EN A</t>
+          <t>EN B</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>26</t>
         </is>
       </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Jako nové (0-50h)</t>
+          <t>Létané (100-200h)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_a</t>
+          <t>paragliding_bazar_cz_b</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN A</t>
+          <t>Paragliding Bazar CZ – EN B</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -35936,21 +36498,23 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Křídlo EN A Advance Alpha 6 26 70-110kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstv Křídlo EN A</t>
+          <t>Křídlo EN B Advance Epsilon DLS 26 Křídlo EN B Advance Epsilon DLS 26 41 225,11 CZK (1 700,00 EUR) EN B Velikost: 26 Opo</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-26-70-110kg-concertinas-no-sivs-no-flyin-7748/</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr"/>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-dls-26-7734/</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>1700</v>
+      </c>
       <c r="G4" t="n">
-        <v>2019</v>
+        <v>2023</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>EN A</t>
+          <t>EN B</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -35961,25 +36525,25 @@
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Jako nové (0-50h)</t>
+          <t>Létané (100-200h)</t>
         </is>
       </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_a</t>
+          <t>paragliding_bazar_cz_b</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN A</t>
+          <t>Paragliding Bazar CZ – EN B</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -35989,38 +36553,93 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Křídlo EN A SKY Paragliders Carancho L 93-116kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN A SK</t>
+          <t>Křídlo EN B MAC Eden 7 26 80-105kg TK čerstvá TK platná Křídlo EN B MAC Eden 7 26 80-105kg TK čerstvá TK platná 18 000,0</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/sky-paragliders-carancho-l-93-116kg-no-sivs-no-flying-on-7746/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/mac-eden-7-26-80-105kg-tc-fresh-tc-valid-7593/</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="n">
-        <v>2005</v>
+        <v>2022</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>EN A</t>
+          <t>EN B</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>26</t>
         </is>
       </c>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Jako nové (0-50h)</t>
+          <t>Létané (100-200h)</t>
         </is>
       </c>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Drift carancho S 69-90kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN A Drift caranch</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/drift-carancho-s-69-90kg-no-sivs-no-flying-on-the-sand-n-7752/</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>1800</v>
+      </c>
+      <c r="G6" t="n">
+        <v>2024</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
         </is>
       </c>
     </row>
@@ -36035,7 +36654,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M3"/>
+  <dimension ref="A1:M4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -36138,7 +36757,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN B Advance Epsilon DLS 26 Křídlo EN B Advance Epsilon DLS 26 41 242,12 CZK (1 700,00 EUR) EN B Velikost: 26 Opo</t>
+          <t>Křídlo EN B Advance Epsilon DLS 26 Křídlo EN B Advance Epsilon DLS 26 41 225,11 CZK (1 700,00 EUR) EN B Velikost: 26 Opo</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -36171,19 +36790,19 @@
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_a</t>
+          <t>paragliding_bazar_cz_b</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN A</t>
+          <t>Paragliding Bazar CZ – EN B</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -36193,38 +36812,93 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Křídlo EN A Gradient Golden 4 24 75-100kg Listovaný Žádné SIV Nelétáno na písku Nekoupáno TK čerstvá Křídlo EN A Gradien</t>
+          <t>Křídlo EN B MAC Eden 7 26 80-105kg TK čerstvá TK platná Křídlo EN B MAC Eden 7 26 80-105kg TK čerstvá TK platná 18 000,0</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/gradient-golden-4-24-75-100kg-concertinas-no-sivs-no-fly-7749/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/mac-eden-7-26-80-105kg-tc-fresh-tc-valid-7593/</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="n">
-        <v>2020</v>
+        <v>2022</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>EN A</t>
+          <t>EN B</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>26</t>
         </is>
       </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Jako nové (0-50h)</t>
+          <t>Létané (100-200h)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Drift carancho S 69-90kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN A Drift caranch</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/drift-carancho-s-69-90kg-no-sivs-no-flying-on-the-sand-n-7752/</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>1800</v>
+      </c>
+      <c r="G4" t="n">
+        <v>2024</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
         </is>
       </c>
     </row>
@@ -36327,12 +37001,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_a</t>
+          <t>paragliding_bazar_cz_b</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN A</t>
+          <t>Paragliding Bazar CZ – EN B</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -36342,38 +37016,38 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN A Gradient Golden 4 24 75-100kg Listovaný Žádné SIV Nelétáno na písku Nekoupáno TK čerstvá Křídlo EN A Gradien</t>
+          <t>Křídlo EN B MAC Eden 7 26 80-105kg TK čerstvá TK platná Křídlo EN B MAC Eden 7 26 80-105kg TK čerstvá TK platná 18 000,0</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/gradient-golden-4-24-75-100kg-concertinas-no-sivs-no-fly-7749/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/mac-eden-7-26-80-105kg-tc-fresh-tc-valid-7593/</t>
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="n">
-        <v>2020</v>
+        <v>2022</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>EN A</t>
+          <t>EN B</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>26</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Jako nové (0-50h)</t>
+          <t>Létané (100-200h)</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: bazar_watcher data update 2026-09-19
</commit_message>
<xml_diff>
--- a/data/bazar_watcher/listings.xlsx
+++ b/data/bazar_watcher/listings.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vsechny inzeraty" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09-2026" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dnes pridane" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Klárka – EN A - low-B, XS-S" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Klárka – EN A - low-B, XXS-XS" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Michal – low-B, S, do 1300 €" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M621"/>
+  <dimension ref="A1:M639"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -34098,8 +34098,10 @@
         </is>
       </c>
       <c r="F617" t="inlineStr"/>
-      <c r="G617" t="n">
-        <v>2015</v>
+      <c r="G617" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
       </c>
       <c r="H617" t="inlineStr">
         <is>
@@ -34150,11 +34152,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/gradient-golden-4-26-85-100kg-tc-fresh-tc-valid-with-lis-7751/</t>
         </is>
       </c>
-      <c r="F618" t="n">
-        <v>620</v>
-      </c>
-      <c r="G618" t="n">
-        <v>2016</v>
+      <c r="F618" t="inlineStr">
+        <is>
+          <t>620.0</t>
+        </is>
+      </c>
+      <c r="G618" t="inlineStr">
+        <is>
+          <t>2016</t>
+        </is>
       </c>
       <c r="H618" t="inlineStr">
         <is>
@@ -34205,11 +34211,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-dls-26-7734/</t>
         </is>
       </c>
-      <c r="F619" t="n">
-        <v>1700</v>
-      </c>
-      <c r="G619" t="n">
-        <v>2023</v>
+      <c r="F619" t="inlineStr">
+        <is>
+          <t>1700.0</t>
+        </is>
+      </c>
+      <c r="G619" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
       </c>
       <c r="H619" t="inlineStr">
         <is>
@@ -34261,8 +34271,10 @@
         </is>
       </c>
       <c r="F620" t="inlineStr"/>
-      <c r="G620" t="n">
-        <v>2022</v>
+      <c r="G620" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
       </c>
       <c r="H620" t="inlineStr">
         <is>
@@ -34313,11 +34325,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/drift-carancho-s-69-90kg-no-sivs-no-flying-on-the-sand-n-7752/</t>
         </is>
       </c>
-      <c r="F621" t="n">
-        <v>1800</v>
-      </c>
-      <c r="G621" t="n">
-        <v>2024</v>
+      <c r="F621" t="inlineStr">
+        <is>
+          <t>1800.0</t>
+        </is>
+      </c>
+      <c r="G621" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
       </c>
       <c r="H621" t="inlineStr">
         <is>
@@ -34339,6 +34355,952 @@
       <c r="M621" t="inlineStr">
         <is>
           <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="622">
+      <c r="A622" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B622" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C622" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D622" t="inlineStr">
+        <is>
+          <t>Křídlo EN B 777 Rook 3 S 70-85kg TK platná Křídlo EN B 777 Rook 3 S 70-85kg TK platná 15 900,00 CZK (650,00 EUR) EN B Ve</t>
+        </is>
+      </c>
+      <c r="E622" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/777-rook-3-s-70-85kg-tc-valid-7800/</t>
+        </is>
+      </c>
+      <c r="F622" t="n">
+        <v>650</v>
+      </c>
+      <c r="G622" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H622" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I622" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J622" t="inlineStr"/>
+      <c r="K622" t="inlineStr">
+        <is>
+          <t>Více létané (200-300h)</t>
+        </is>
+      </c>
+      <c r="L622" t="inlineStr"/>
+      <c r="M622" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="623">
+      <c r="A623" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B623" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C623" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D623" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AirDesign Susi 3 21 60-108kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B AirDesign</t>
+        </is>
+      </c>
+      <c r="E623" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/airdesign-susi-3-21-60-108kg-no-sivs-no-flying-on-the-sa-7799/</t>
+        </is>
+      </c>
+      <c r="F623" t="n">
+        <v>1500</v>
+      </c>
+      <c r="G623" t="n">
+        <v>2021</v>
+      </c>
+      <c r="H623" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I623" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="J623" t="inlineStr"/>
+      <c r="K623" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L623" t="inlineStr"/>
+      <c r="M623" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="624">
+      <c r="A624" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B624" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C624" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D624" t="inlineStr">
+        <is>
+          <t>Křídlo EN B UP Kibo M 75-95kg Listovaný Žádné SIV Nevětveno Nekoupáno TK platná Křídlo EN B UP Kibo M 75-95kg Listovaný</t>
+        </is>
+      </c>
+      <c r="E624" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/up-kibo-m-75-95kg-concertinas-no-sivs-no-trees-no-water--7798/</t>
+        </is>
+      </c>
+      <c r="F624" t="inlineStr"/>
+      <c r="G624" t="n">
+        <v>2018</v>
+      </c>
+      <c r="H624" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I624" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J624" t="inlineStr"/>
+      <c r="K624" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L624" t="inlineStr"/>
+      <c r="M624" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="625">
+      <c r="A625" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B625" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C625" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D625" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Gradient Golden 4 26 85-100kg Žádné SIV Nelétáno na písku Nevětveno TK platná Křídlo EN B Gradient Golden 4</t>
+        </is>
+      </c>
+      <c r="E625" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/gradient-golden-4-26-85-100kg-no-sivs-no-flying-on-the-s-7788/</t>
+        </is>
+      </c>
+      <c r="F625" t="inlineStr"/>
+      <c r="G625" t="n">
+        <v>2013</v>
+      </c>
+      <c r="H625" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I625" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="J625" t="inlineStr"/>
+      <c r="K625" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L625" t="inlineStr"/>
+      <c r="M625" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="626">
+      <c r="A626" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B626" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C626" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D626" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Skyman Crosscountry 2 M 80-105kg Křídlo EN B Skyman Crosscountry 2 M 80-105kg 24 000,00 CZK EN B Velikost: M</t>
+        </is>
+      </c>
+      <c r="E626" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/skyman-crosscountry-2-m-80-105kg-7776/</t>
+        </is>
+      </c>
+      <c r="F626" t="inlineStr"/>
+      <c r="G626" t="n">
+        <v>2019</v>
+      </c>
+      <c r="H626" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I626" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J626" t="inlineStr"/>
+      <c r="K626" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L626" t="inlineStr"/>
+      <c r="M626" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="627">
+      <c r="A627" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B627" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C627" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D627" t="inlineStr">
+        <is>
+          <t>Křídlo EN B SKY Paragliders Kudos 2 L 85-108kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá Křídlo EN B SK</t>
+        </is>
+      </c>
+      <c r="E627" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/sky-paragliders-kudos-2-l-85-108kg-no-sivs-no-flying-on--7764/</t>
+        </is>
+      </c>
+      <c r="F627" t="inlineStr"/>
+      <c r="G627" t="n">
+        <v>2024</v>
+      </c>
+      <c r="H627" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I627" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J627" t="inlineStr"/>
+      <c r="K627" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L627" t="inlineStr"/>
+      <c r="M627" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="628">
+      <c r="A628" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B628" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C628" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D628" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AXIS Pluto 3 ML 95-115kg Křídlo EN B AXIS Pluto 3 ML 95-115kg 7 500,00 CZK EN B Velikost: ML Vzletová hmotno</t>
+        </is>
+      </c>
+      <c r="E628" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-pluto-3-ml-95-115kg-7763/</t>
+        </is>
+      </c>
+      <c r="F628" t="inlineStr"/>
+      <c r="G628" t="n">
+        <v>2016</v>
+      </c>
+      <c r="H628" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I628" t="inlineStr">
+        <is>
+          <t>ML</t>
+        </is>
+      </c>
+      <c r="J628" t="inlineStr"/>
+      <c r="K628" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L628" t="inlineStr"/>
+      <c r="M628" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="629">
+      <c r="A629" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B629" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C629" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D629" t="inlineStr">
+        <is>
+          <t>Křídlo EN B UP SUMMIT X M 85-110kg Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B UP SUMMIT X M 85-110kg Ne</t>
+        </is>
+      </c>
+      <c r="E629" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/up-summit-x-m-85-110kg-no-flying-on-the-sand-no-trees-no-7762/</t>
+        </is>
+      </c>
+      <c r="F629" t="inlineStr"/>
+      <c r="G629" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H629" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I629" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J629" t="inlineStr"/>
+      <c r="K629" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L629" t="inlineStr"/>
+      <c r="M629" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="630">
+      <c r="A630" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B630" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C630" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D630" t="inlineStr">
+        <is>
+          <t>Křídlo EN B MAC Eden8 100-130kg Listovaný Žádné SIV Nelétáno na písku Nevětveno TK platná Křídlo EN B MAC Eden8 100-130k</t>
+        </is>
+      </c>
+      <c r="E630" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/mac-eden8-100-130kg-concertinas-no-sivs-no-flying-on-the-7761/</t>
+        </is>
+      </c>
+      <c r="F630" t="inlineStr"/>
+      <c r="G630" t="n">
+        <v>2026</v>
+      </c>
+      <c r="H630" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I630" t="inlineStr"/>
+      <c r="J630" t="inlineStr"/>
+      <c r="K630" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L630" t="inlineStr"/>
+      <c r="M630" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="631">
+      <c r="A631" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B631" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C631" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D631" t="inlineStr">
+        <is>
+          <t>Křídlo EN B SKY Paragliders Kudos 2 L 85-110kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Křídlo EN B SKY</t>
+        </is>
+      </c>
+      <c r="E631" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/sky-paragliders-kudos-2-l-85-110kg-concertinas-no-sivs-n-7756/</t>
+        </is>
+      </c>
+      <c r="F631" t="n">
+        <v>2900</v>
+      </c>
+      <c r="G631" t="n">
+        <v>2025</v>
+      </c>
+      <c r="H631" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I631" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J631" t="inlineStr"/>
+      <c r="K631" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L631" t="inlineStr"/>
+      <c r="M631" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="632">
+      <c r="A632" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B632" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C632" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D632" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AXIS Comet 3 M Listovaný Nové Žádné SIV Křídlo EN B AXIS Comet 3 M Listovaný Nové Žádné SIV 21 834,06 CZK (9</t>
+        </is>
+      </c>
+      <c r="E632" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-concertinas-new-no-sivs-7529/</t>
+        </is>
+      </c>
+      <c r="F632" t="n">
+        <v>900</v>
+      </c>
+      <c r="G632" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H632" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I632" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J632" t="inlineStr"/>
+      <c r="K632" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L632" t="inlineStr"/>
+      <c r="M632" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="633">
+      <c r="A633" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B633" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C633" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D633" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Nova Prion 5 M 90-115kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN A Nova</t>
+        </is>
+      </c>
+      <c r="E633" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-prion-5-m-90-115kg-concertinas-no-sivs-no-flying-on-7790/</t>
+        </is>
+      </c>
+      <c r="F633" t="n">
+        <v>1200</v>
+      </c>
+      <c r="G633" t="n">
+        <v>2022</v>
+      </c>
+      <c r="H633" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I633" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J633" t="inlineStr"/>
+      <c r="K633" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L633" t="inlineStr"/>
+      <c r="M633" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="634">
+      <c r="A634" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B634" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C634" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D634" t="inlineStr">
+        <is>
+          <t>Křídlo EN A MAC Lucky 4 28 85-110kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Drobné opravy TK platná Křídlo EN A</t>
+        </is>
+      </c>
+      <c r="E634" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/mac-lucky-4-28-85-110kg-no-sivs-no-flying-on-the-sand-no-7789/</t>
+        </is>
+      </c>
+      <c r="F634" t="inlineStr"/>
+      <c r="G634" t="n">
+        <v>2016</v>
+      </c>
+      <c r="H634" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I634" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J634" t="inlineStr"/>
+      <c r="K634" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L634" t="inlineStr"/>
+      <c r="M634" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="635">
+      <c r="A635" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B635" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C635" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D635" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Gradient Bright 5 26 75-100kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá Křídlo EN A Gradien</t>
+        </is>
+      </c>
+      <c r="E635" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/gradient-bright-5-26-75-100kg-no-sivs-no-flying-on-the-s-7787/</t>
+        </is>
+      </c>
+      <c r="F635" t="inlineStr"/>
+      <c r="G635" t="n">
+        <v>2018</v>
+      </c>
+      <c r="H635" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I635" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="J635" t="inlineStr"/>
+      <c r="K635" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L635" t="inlineStr"/>
+      <c r="M635" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="636">
+      <c r="A636" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B636" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C636" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D636" t="inlineStr">
+        <is>
+          <t>Křídlo EN A MAC Lucky 4 30 105-130kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá (Součást kompl</t>
+        </is>
+      </c>
+      <c r="E636" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/mac-lucky-4-30-105-130kg-concertinas-no-sivs-no-flying-o-7780/</t>
+        </is>
+      </c>
+      <c r="F636" t="n">
+        <v>1600</v>
+      </c>
+      <c r="G636" t="n">
+        <v>2022</v>
+      </c>
+      <c r="H636" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I636" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="J636" t="inlineStr"/>
+      <c r="K636" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L636" t="inlineStr"/>
+      <c r="M636" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="637">
+      <c r="A637" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B637" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C637" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D637" t="inlineStr">
+        <is>
+          <t>Křídlo EN A SKY Paragliders Gaia3M M 73-97kg Listovaný Nové Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Křídlo EN A</t>
+        </is>
+      </c>
+      <c r="E637" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/sky-paragliders-gaia3m-m-73-97kg-concertinas-new-no-sivs-7769/</t>
+        </is>
+      </c>
+      <c r="F637" t="inlineStr"/>
+      <c r="G637" t="n">
+        <v>2026</v>
+      </c>
+      <c r="H637" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I637" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J637" t="inlineStr"/>
+      <c r="K637" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L637" t="inlineStr"/>
+      <c r="M637" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="638">
+      <c r="A638" t="inlineStr">
+        <is>
+          <t>hochries_de</t>
+        </is>
+      </c>
+      <c r="B638" t="inlineStr">
+        <is>
+          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
+        </is>
+      </c>
+      <c r="C638" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D638" t="inlineStr">
+        <is>
+          <t>AIRDESIGN Volt 5 M</t>
+        </is>
+      </c>
+      <c r="E638" t="inlineStr">
+        <is>
+          <t>https://shop.flugschule-hochries.de/AIRDESIGN-Volt-5-M/SW10612</t>
+        </is>
+      </c>
+      <c r="F638" t="n">
+        <v>3000</v>
+      </c>
+      <c r="G638" t="inlineStr"/>
+      <c r="H638" t="inlineStr"/>
+      <c r="I638" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J638" t="inlineStr"/>
+      <c r="K638" t="inlineStr"/>
+      <c r="L638" t="inlineStr"/>
+      <c r="M638" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="639">
+      <c r="A639" t="inlineStr">
+        <is>
+          <t>hochries_de</t>
+        </is>
+      </c>
+      <c r="B639" t="inlineStr">
+        <is>
+          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
+        </is>
+      </c>
+      <c r="C639" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D639" t="inlineStr">
+        <is>
+          <t>AIRDESIGN Volt 5 S</t>
+        </is>
+      </c>
+      <c r="E639" t="inlineStr">
+        <is>
+          <t>https://shop.flugschule-hochries.de/AIRDESIGN-Volt-5-S/SW10610</t>
+        </is>
+      </c>
+      <c r="F639" t="n">
+        <v>3650</v>
+      </c>
+      <c r="G639" t="inlineStr"/>
+      <c r="H639" t="inlineStr"/>
+      <c r="I639" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J639" t="inlineStr"/>
+      <c r="K639" t="inlineStr"/>
+      <c r="L639" t="inlineStr"/>
+      <c r="M639" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
         </is>
       </c>
     </row>
@@ -34353,11 +35315,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M35"/>
+  <dimension ref="A1:M53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
@@ -36032,8 +36994,10 @@
         </is>
       </c>
       <c r="F31" t="inlineStr"/>
-      <c r="G31" t="n">
-        <v>2015</v>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
@@ -36084,11 +37048,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/gradient-golden-4-26-85-100kg-tc-fresh-tc-valid-with-lis-7751/</t>
         </is>
       </c>
-      <c r="F32" t="n">
-        <v>620</v>
-      </c>
-      <c r="G32" t="n">
-        <v>2016</v>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>620.0</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>2016</t>
+        </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
@@ -36139,11 +37107,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-dls-26-7734/</t>
         </is>
       </c>
-      <c r="F33" t="n">
-        <v>1700</v>
-      </c>
-      <c r="G33" t="n">
-        <v>2023</v>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>1700.0</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
@@ -36195,8 +37167,10 @@
         </is>
       </c>
       <c r="F34" t="inlineStr"/>
-      <c r="G34" t="n">
-        <v>2022</v>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
@@ -36247,11 +37221,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/drift-carancho-s-69-90kg-no-sivs-no-flying-on-the-sand-n-7752/</t>
         </is>
       </c>
-      <c r="F35" t="n">
-        <v>1800</v>
-      </c>
-      <c r="G35" t="n">
-        <v>2024</v>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>1800.0</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
@@ -36273,6 +37251,952 @@
       <c r="M35" t="inlineStr">
         <is>
           <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Křídlo EN B 777 Rook 3 S 70-85kg TK platná Křídlo EN B 777 Rook 3 S 70-85kg TK platná 15 900,00 CZK (650,00 EUR) EN B Ve</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/777-rook-3-s-70-85kg-tc-valid-7800/</t>
+        </is>
+      </c>
+      <c r="F36" t="n">
+        <v>650</v>
+      </c>
+      <c r="G36" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr"/>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>Více létané (200-300h)</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr"/>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AirDesign Susi 3 21 60-108kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B AirDesign</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/airdesign-susi-3-21-60-108kg-no-sivs-no-flying-on-the-sa-7799/</t>
+        </is>
+      </c>
+      <c r="F37" t="n">
+        <v>1500</v>
+      </c>
+      <c r="G37" t="n">
+        <v>2021</v>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr"/>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr"/>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Křídlo EN B UP Kibo M 75-95kg Listovaný Žádné SIV Nevětveno Nekoupáno TK platná Křídlo EN B UP Kibo M 75-95kg Listovaný</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/up-kibo-m-75-95kg-concertinas-no-sivs-no-trees-no-water--7798/</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr"/>
+      <c r="G38" t="n">
+        <v>2018</v>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr"/>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr"/>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Gradient Golden 4 26 85-100kg Žádné SIV Nelétáno na písku Nevětveno TK platná Křídlo EN B Gradient Golden 4</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/gradient-golden-4-26-85-100kg-no-sivs-no-flying-on-the-s-7788/</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr"/>
+      <c r="G39" t="n">
+        <v>2013</v>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr"/>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr"/>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Skyman Crosscountry 2 M 80-105kg Křídlo EN B Skyman Crosscountry 2 M 80-105kg 24 000,00 CZK EN B Velikost: M</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/skyman-crosscountry-2-m-80-105kg-7776/</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr"/>
+      <c r="G40" t="n">
+        <v>2019</v>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr"/>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr"/>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Křídlo EN B SKY Paragliders Kudos 2 L 85-108kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá Křídlo EN B SK</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/sky-paragliders-kudos-2-l-85-108kg-no-sivs-no-flying-on--7764/</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr"/>
+      <c r="G41" t="n">
+        <v>2024</v>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr"/>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr"/>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AXIS Pluto 3 ML 95-115kg Křídlo EN B AXIS Pluto 3 ML 95-115kg 7 500,00 CZK EN B Velikost: ML Vzletová hmotno</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-pluto-3-ml-95-115kg-7763/</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr"/>
+      <c r="G42" t="n">
+        <v>2016</v>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>ML</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr"/>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr"/>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Křídlo EN B UP SUMMIT X M 85-110kg Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B UP SUMMIT X M 85-110kg Ne</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/up-summit-x-m-85-110kg-no-flying-on-the-sand-no-trees-no-7762/</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr"/>
+      <c r="G43" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr"/>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr"/>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Křídlo EN B MAC Eden8 100-130kg Listovaný Žádné SIV Nelétáno na písku Nevětveno TK platná Křídlo EN B MAC Eden8 100-130k</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/mac-eden8-100-130kg-concertinas-no-sivs-no-flying-on-the-7761/</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr"/>
+      <c r="G44" t="n">
+        <v>2026</v>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr"/>
+      <c r="J44" t="inlineStr"/>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr"/>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Křídlo EN B SKY Paragliders Kudos 2 L 85-110kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Křídlo EN B SKY</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/sky-paragliders-kudos-2-l-85-110kg-concertinas-no-sivs-n-7756/</t>
+        </is>
+      </c>
+      <c r="F45" t="n">
+        <v>2900</v>
+      </c>
+      <c r="G45" t="n">
+        <v>2025</v>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr"/>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr"/>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AXIS Comet 3 M Listovaný Nové Žádné SIV Křídlo EN B AXIS Comet 3 M Listovaný Nové Žádné SIV 21 834,06 CZK (9</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-concertinas-new-no-sivs-7529/</t>
+        </is>
+      </c>
+      <c r="F46" t="n">
+        <v>900</v>
+      </c>
+      <c r="G46" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr"/>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr"/>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Nova Prion 5 M 90-115kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN A Nova</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-prion-5-m-90-115kg-concertinas-no-sivs-no-flying-on-7790/</t>
+        </is>
+      </c>
+      <c r="F47" t="n">
+        <v>1200</v>
+      </c>
+      <c r="G47" t="n">
+        <v>2022</v>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr"/>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr"/>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Křídlo EN A MAC Lucky 4 28 85-110kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Drobné opravy TK platná Křídlo EN A</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/mac-lucky-4-28-85-110kg-no-sivs-no-flying-on-the-sand-no-7789/</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr"/>
+      <c r="G48" t="n">
+        <v>2016</v>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr"/>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr"/>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Gradient Bright 5 26 75-100kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá Křídlo EN A Gradien</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/gradient-bright-5-26-75-100kg-no-sivs-no-flying-on-the-s-7787/</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr"/>
+      <c r="G49" t="n">
+        <v>2018</v>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr"/>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr"/>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Křídlo EN A MAC Lucky 4 30 105-130kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá (Součást kompl</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/mac-lucky-4-30-105-130kg-concertinas-no-sivs-no-flying-o-7780/</t>
+        </is>
+      </c>
+      <c r="F50" t="n">
+        <v>1600</v>
+      </c>
+      <c r="G50" t="n">
+        <v>2022</v>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr"/>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr"/>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Křídlo EN A SKY Paragliders Gaia3M M 73-97kg Listovaný Nové Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Křídlo EN A</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/sky-paragliders-gaia3m-m-73-97kg-concertinas-new-no-sivs-7769/</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr"/>
+      <c r="G51" t="n">
+        <v>2026</v>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr"/>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr"/>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>hochries_de</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>AIRDESIGN Volt 5 M</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>https://shop.flugschule-hochries.de/AIRDESIGN-Volt-5-M/SW10612</t>
+        </is>
+      </c>
+      <c r="F52" t="n">
+        <v>3000</v>
+      </c>
+      <c r="G52" t="inlineStr"/>
+      <c r="H52" t="inlineStr"/>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr"/>
+      <c r="K52" t="inlineStr"/>
+      <c r="L52" t="inlineStr"/>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>hochries_de</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>AIRDESIGN Volt 5 S</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>https://shop.flugschule-hochries.de/AIRDESIGN-Volt-5-S/SW10610</t>
+        </is>
+      </c>
+      <c r="F53" t="n">
+        <v>3650</v>
+      </c>
+      <c r="G53" t="inlineStr"/>
+      <c r="H53" t="inlineStr"/>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr"/>
+      <c r="K53" t="inlineStr"/>
+      <c r="L53" t="inlineStr"/>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
         </is>
       </c>
     </row>
@@ -36287,20 +38211,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M6"/>
+  <dimension ref="A1:M19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="25" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
@@ -36390,17 +38314,19 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN B Ozone Buzz z4 S 65-85kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B Ozon</t>
+          <t>Křídlo EN B 777 Rook 3 S 70-85kg TK platná Křídlo EN B 777 Rook 3 S 70-85kg TK platná 15 900,00 CZK (650,00 EUR) EN B Ve</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/ozone-buzz-z4-s-65-85kg-concertinas-no-sivs-no-flying-on-7753/</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
+          <t>https://paragliding-bazar.cz/cs/offering/777-rook-3-s-70-85kg-tc-valid-7800/</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>650</v>
+      </c>
       <c r="G2" t="n">
-        <v>2015</v>
+        <v>2020</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -36415,13 +38341,13 @@
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Jako nové (0-50h)</t>
+          <t>Více létané (200-300h)</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-19</t>
         </is>
       </c>
     </row>
@@ -36443,19 +38369,19 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Křídlo EN B Gradient Golden 4 26 85-100kg TK čerstvá TK platná S listovacím obalem Křídlo EN B Gradient Golden 4 26 85-1</t>
+          <t>Křídlo EN B AirDesign Susi 3 21 60-108kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B AirDesign</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/gradient-golden-4-26-85-100kg-tc-fresh-tc-valid-with-lis-7751/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/airdesign-susi-3-21-60-108kg-no-sivs-no-flying-on-the-sa-7799/</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>620</v>
+        <v>1500</v>
       </c>
       <c r="G3" t="n">
-        <v>2016</v>
+        <v>2021</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -36464,19 +38390,19 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Létané (100-200h)</t>
+          <t>Jako nové (0-50h)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-19</t>
         </is>
       </c>
     </row>
@@ -36498,19 +38424,17 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Křídlo EN B Advance Epsilon DLS 26 Křídlo EN B Advance Epsilon DLS 26 41 225,11 CZK (1 700,00 EUR) EN B Velikost: 26 Opo</t>
+          <t>Křídlo EN B UP Kibo M 75-95kg Listovaný Žádné SIV Nevětveno Nekoupáno TK platná Křídlo EN B UP Kibo M 75-95kg Listovaný</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-dls-26-7734/</t>
-        </is>
-      </c>
-      <c r="F4" t="n">
-        <v>1700</v>
-      </c>
+          <t>https://paragliding-bazar.cz/cs/offering/up-kibo-m-75-95kg-concertinas-no-sivs-no-trees-no-water--7798/</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
       <c r="G4" t="n">
-        <v>2023</v>
+        <v>2018</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -36519,7 +38443,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>M</t>
         </is>
       </c>
       <c r="J4" t="inlineStr"/>
@@ -36531,7 +38455,7 @@
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-19</t>
         </is>
       </c>
     </row>
@@ -36553,17 +38477,17 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Křídlo EN B MAC Eden 7 26 80-105kg TK čerstvá TK platná Křídlo EN B MAC Eden 7 26 80-105kg TK čerstvá TK platná 18 000,0</t>
+          <t>Křídlo EN B Gradient Golden 4 26 85-100kg Žádné SIV Nelétáno na písku Nevětveno TK platná Křídlo EN B Gradient Golden 4</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/mac-eden-7-26-80-105kg-tc-fresh-tc-valid-7593/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/gradient-golden-4-26-85-100kg-no-sivs-no-flying-on-the-s-7788/</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="n">
-        <v>2022</v>
+        <v>2013</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -36578,25 +38502,25 @@
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Létané (100-200h)</t>
+          <t>Mírně létané (50-100h)</t>
         </is>
       </c>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-19</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_a</t>
+          <t>paragliding_bazar_cz_b</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN A</t>
+          <t>Paragliding Bazar CZ – EN B</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -36606,40 +38530,715 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Křídlo EN A Drift carancho S 69-90kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN A Drift caranch</t>
+          <t>Křídlo EN B Skyman Crosscountry 2 M 80-105kg Křídlo EN B Skyman Crosscountry 2 M 80-105kg 24 000,00 CZK EN B Velikost: M</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/drift-carancho-s-69-90kg-no-sivs-no-flying-on-the-sand-n-7752/</t>
-        </is>
-      </c>
-      <c r="F6" t="n">
-        <v>1800</v>
-      </c>
+          <t>https://paragliding-bazar.cz/cs/offering/skyman-crosscountry-2-m-80-105kg-7776/</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
       <c r="G6" t="n">
-        <v>2024</v>
+        <v>2019</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>EN A</t>
+          <t>EN B</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Jako nové (0-50h)</t>
+          <t>Létané (100-200h)</t>
         </is>
       </c>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Křídlo EN B SKY Paragliders Kudos 2 L 85-108kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá Křídlo EN B SK</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/sky-paragliders-kudos-2-l-85-108kg-no-sivs-no-flying-on--7764/</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="n">
+        <v>2024</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AXIS Pluto 3 ML 95-115kg Křídlo EN B AXIS Pluto 3 ML 95-115kg 7 500,00 CZK EN B Velikost: ML Vzletová hmotno</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-pluto-3-ml-95-115kg-7763/</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="n">
+        <v>2016</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>ML</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Křídlo EN B UP SUMMIT X M 85-110kg Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B UP SUMMIT X M 85-110kg Ne</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/up-summit-x-m-85-110kg-no-flying-on-the-sand-no-trees-no-7762/</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Křídlo EN B MAC Eden8 100-130kg Listovaný Žádné SIV Nelétáno na písku Nevětveno TK platná Křídlo EN B MAC Eden8 100-130k</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/mac-eden8-100-130kg-concertinas-no-sivs-no-flying-on-the-7761/</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="n">
+        <v>2026</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Křídlo EN B SKY Paragliders Kudos 2 L 85-110kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Křídlo EN B SKY</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/sky-paragliders-kudos-2-l-85-110kg-concertinas-no-sivs-n-7756/</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>2900</v>
+      </c>
+      <c r="G11" t="n">
+        <v>2025</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AXIS Comet 3 M Listovaný Nové Žádné SIV Křídlo EN B AXIS Comet 3 M Listovaný Nové Žádné SIV 21 834,06 CZK (9</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-concertinas-new-no-sivs-7529/</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>900</v>
+      </c>
+      <c r="G12" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Nova Prion 5 M 90-115kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN A Nova</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-prion-5-m-90-115kg-concertinas-no-sivs-no-flying-on-7790/</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>1200</v>
+      </c>
+      <c r="G13" t="n">
+        <v>2022</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Křídlo EN A MAC Lucky 4 28 85-110kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Drobné opravy TK platná Křídlo EN A</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/mac-lucky-4-28-85-110kg-no-sivs-no-flying-on-the-sand-no-7789/</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="n">
+        <v>2016</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Křídlo EN A Gradient Bright 5 26 75-100kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá Křídlo EN A Gradien</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/gradient-bright-5-26-75-100kg-no-sivs-no-flying-on-the-s-7787/</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="n">
+        <v>2018</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Křídlo EN A MAC Lucky 4 30 105-130kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá (Součást kompl</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/mac-lucky-4-30-105-130kg-concertinas-no-sivs-no-flying-o-7780/</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>1600</v>
+      </c>
+      <c r="G16" t="n">
+        <v>2022</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Křídlo EN A SKY Paragliders Gaia3M M 73-97kg Listovaný Nové Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Křídlo EN A</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/sky-paragliders-gaia3m-m-73-97kg-concertinas-new-no-sivs-7769/</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="n">
+        <v>2026</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>hochries_de</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>AIRDESIGN Volt 5 M</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>https://shop.flugschule-hochries.de/AIRDESIGN-Volt-5-M/SW10612</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>3000</v>
+      </c>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>hochries_de</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>AIRDESIGN Volt 5 S</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>https://shop.flugschule-hochries.de/AIRDESIGN-Volt-5-S/SW10610</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>3650</v>
+      </c>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
         </is>
       </c>
     </row>
@@ -36654,20 +39253,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M4"/>
+  <dimension ref="A1:M5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="25" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
@@ -36757,19 +39356,19 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN B Advance Epsilon DLS 26 Křídlo EN B Advance Epsilon DLS 26 41 225,11 CZK (1 700,00 EUR) EN B Velikost: 26 Opo</t>
+          <t>Křídlo EN B 777 Rook 3 S 70-85kg TK platná Křídlo EN B 777 Rook 3 S 70-85kg TK platná 15 900,00 CZK (650,00 EUR) EN B Ve</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-dls-26-7734/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/777-rook-3-s-70-85kg-tc-valid-7800/</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>1700</v>
+        <v>650</v>
       </c>
       <c r="G2" t="n">
-        <v>2023</v>
+        <v>2020</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -36778,19 +39377,19 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>S</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Létané (100-200h)</t>
+          <t>Více létané (200-300h)</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-19</t>
         </is>
       </c>
     </row>
@@ -36812,17 +39411,19 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Křídlo EN B MAC Eden 7 26 80-105kg TK čerstvá TK platná Křídlo EN B MAC Eden 7 26 80-105kg TK čerstvá TK platná 18 000,0</t>
+          <t>Křídlo EN B AirDesign Susi 3 21 60-108kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B AirDesign</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/mac-eden-7-26-80-105kg-tc-fresh-tc-valid-7593/</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
+          <t>https://paragliding-bazar.cz/cs/offering/airdesign-susi-3-21-60-108kg-no-sivs-no-flying-on-the-sa-7799/</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>1500</v>
+      </c>
       <c r="G3" t="n">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -36831,31 +39432,31 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Létané (100-200h)</t>
+          <t>Jako nové (0-50h)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-19</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_a</t>
+          <t>paragliding_bazar_cz_b</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN A</t>
+          <t>Paragliding Bazar CZ – EN B</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -36865,28 +39466,28 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Křídlo EN A Drift carancho S 69-90kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN A Drift caranch</t>
+          <t>Křídlo EN B AXIS Comet 3 M Listovaný Nové Žádné SIV Křídlo EN B AXIS Comet 3 M Listovaný Nové Žádné SIV 21 834,06 CZK (9</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/drift-carancho-s-69-90kg-no-sivs-no-flying-on-the-sand-n-7752/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-concertinas-new-no-sivs-7529/</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>1800</v>
+        <v>900</v>
       </c>
       <c r="G4" t="n">
-        <v>2024</v>
+        <v>2020</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>EN A</t>
+          <t>EN B</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="J4" t="inlineStr"/>
@@ -36898,7 +39499,52 @@
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>hochries_de</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>AIRDESIGN Volt 5 S</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>https://shop.flugschule-hochries.de/AIRDESIGN-Volt-5-S/SW10610</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>3650</v>
+      </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
         </is>
       </c>
     </row>
@@ -36926,7 +39572,7 @@
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="25" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
@@ -37016,17 +39662,19 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN B MAC Eden 7 26 80-105kg TK čerstvá TK platná Křídlo EN B MAC Eden 7 26 80-105kg TK čerstvá TK platná 18 000,0</t>
+          <t>Křídlo EN B 777 Rook 3 S 70-85kg TK platná Křídlo EN B 777 Rook 3 S 70-85kg TK platná 15 900,00 CZK (650,00 EUR) EN B Ve</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/mac-eden-7-26-80-105kg-tc-fresh-tc-valid-7593/</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
+          <t>https://paragliding-bazar.cz/cs/offering/777-rook-3-s-70-85kg-tc-valid-7800/</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>650</v>
+      </c>
       <c r="G2" t="n">
-        <v>2022</v>
+        <v>2020</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -37035,19 +39683,19 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>S</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Létané (100-200h)</t>
+          <t>Více létané (200-300h)</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-19</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: bazar_watcher data update 2026-09-26
</commit_message>
<xml_diff>
--- a/data/bazar_watcher/listings.xlsx
+++ b/data/bazar_watcher/listings.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M639"/>
+  <dimension ref="A1:M649"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -34384,11 +34384,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/777-rook-3-s-70-85kg-tc-valid-7800/</t>
         </is>
       </c>
-      <c r="F622" t="n">
-        <v>650</v>
-      </c>
-      <c r="G622" t="n">
-        <v>2020</v>
+      <c r="F622" t="inlineStr">
+        <is>
+          <t>650.0</t>
+        </is>
+      </c>
+      <c r="G622" t="inlineStr">
+        <is>
+          <t>2020.0</t>
+        </is>
       </c>
       <c r="H622" t="inlineStr">
         <is>
@@ -34439,11 +34443,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/airdesign-susi-3-21-60-108kg-no-sivs-no-flying-on-the-sa-7799/</t>
         </is>
       </c>
-      <c r="F623" t="n">
-        <v>1500</v>
-      </c>
-      <c r="G623" t="n">
-        <v>2021</v>
+      <c r="F623" t="inlineStr">
+        <is>
+          <t>1500.0</t>
+        </is>
+      </c>
+      <c r="G623" t="inlineStr">
+        <is>
+          <t>2021.0</t>
+        </is>
       </c>
       <c r="H623" t="inlineStr">
         <is>
@@ -34495,8 +34503,10 @@
         </is>
       </c>
       <c r="F624" t="inlineStr"/>
-      <c r="G624" t="n">
-        <v>2018</v>
+      <c r="G624" t="inlineStr">
+        <is>
+          <t>2018.0</t>
+        </is>
       </c>
       <c r="H624" t="inlineStr">
         <is>
@@ -34548,8 +34558,10 @@
         </is>
       </c>
       <c r="F625" t="inlineStr"/>
-      <c r="G625" t="n">
-        <v>2013</v>
+      <c r="G625" t="inlineStr">
+        <is>
+          <t>2013.0</t>
+        </is>
       </c>
       <c r="H625" t="inlineStr">
         <is>
@@ -34601,8 +34613,10 @@
         </is>
       </c>
       <c r="F626" t="inlineStr"/>
-      <c r="G626" t="n">
-        <v>2019</v>
+      <c r="G626" t="inlineStr">
+        <is>
+          <t>2019.0</t>
+        </is>
       </c>
       <c r="H626" t="inlineStr">
         <is>
@@ -34654,8 +34668,10 @@
         </is>
       </c>
       <c r="F627" t="inlineStr"/>
-      <c r="G627" t="n">
-        <v>2024</v>
+      <c r="G627" t="inlineStr">
+        <is>
+          <t>2024.0</t>
+        </is>
       </c>
       <c r="H627" t="inlineStr">
         <is>
@@ -34707,8 +34723,10 @@
         </is>
       </c>
       <c r="F628" t="inlineStr"/>
-      <c r="G628" t="n">
-        <v>2016</v>
+      <c r="G628" t="inlineStr">
+        <is>
+          <t>2016.0</t>
+        </is>
       </c>
       <c r="H628" t="inlineStr">
         <is>
@@ -34760,8 +34778,10 @@
         </is>
       </c>
       <c r="F629" t="inlineStr"/>
-      <c r="G629" t="n">
-        <v>2023</v>
+      <c r="G629" t="inlineStr">
+        <is>
+          <t>2023.0</t>
+        </is>
       </c>
       <c r="H629" t="inlineStr">
         <is>
@@ -34813,8 +34833,10 @@
         </is>
       </c>
       <c r="F630" t="inlineStr"/>
-      <c r="G630" t="n">
-        <v>2026</v>
+      <c r="G630" t="inlineStr">
+        <is>
+          <t>2026.0</t>
+        </is>
       </c>
       <c r="H630" t="inlineStr">
         <is>
@@ -34861,11 +34883,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/sky-paragliders-kudos-2-l-85-110kg-concertinas-no-sivs-n-7756/</t>
         </is>
       </c>
-      <c r="F631" t="n">
-        <v>2900</v>
-      </c>
-      <c r="G631" t="n">
-        <v>2025</v>
+      <c r="F631" t="inlineStr">
+        <is>
+          <t>2900.0</t>
+        </is>
+      </c>
+      <c r="G631" t="inlineStr">
+        <is>
+          <t>2025.0</t>
+        </is>
       </c>
       <c r="H631" t="inlineStr">
         <is>
@@ -34916,11 +34942,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-concertinas-new-no-sivs-7529/</t>
         </is>
       </c>
-      <c r="F632" t="n">
-        <v>900</v>
-      </c>
-      <c r="G632" t="n">
-        <v>2020</v>
+      <c r="F632" t="inlineStr">
+        <is>
+          <t>900.0</t>
+        </is>
+      </c>
+      <c r="G632" t="inlineStr">
+        <is>
+          <t>2020.0</t>
+        </is>
       </c>
       <c r="H632" t="inlineStr">
         <is>
@@ -34971,11 +35001,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/nova-prion-5-m-90-115kg-concertinas-no-sivs-no-flying-on-7790/</t>
         </is>
       </c>
-      <c r="F633" t="n">
-        <v>1200</v>
-      </c>
-      <c r="G633" t="n">
-        <v>2022</v>
+      <c r="F633" t="inlineStr">
+        <is>
+          <t>1200.0</t>
+        </is>
+      </c>
+      <c r="G633" t="inlineStr">
+        <is>
+          <t>2022.0</t>
+        </is>
       </c>
       <c r="H633" t="inlineStr">
         <is>
@@ -35027,8 +35061,10 @@
         </is>
       </c>
       <c r="F634" t="inlineStr"/>
-      <c r="G634" t="n">
-        <v>2016</v>
+      <c r="G634" t="inlineStr">
+        <is>
+          <t>2016.0</t>
+        </is>
       </c>
       <c r="H634" t="inlineStr">
         <is>
@@ -35080,8 +35116,10 @@
         </is>
       </c>
       <c r="F635" t="inlineStr"/>
-      <c r="G635" t="n">
-        <v>2018</v>
+      <c r="G635" t="inlineStr">
+        <is>
+          <t>2018.0</t>
+        </is>
       </c>
       <c r="H635" t="inlineStr">
         <is>
@@ -35132,11 +35170,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/mac-lucky-4-30-105-130kg-concertinas-no-sivs-no-flying-o-7780/</t>
         </is>
       </c>
-      <c r="F636" t="n">
-        <v>1600</v>
-      </c>
-      <c r="G636" t="n">
-        <v>2022</v>
+      <c r="F636" t="inlineStr">
+        <is>
+          <t>1600.0</t>
+        </is>
+      </c>
+      <c r="G636" t="inlineStr">
+        <is>
+          <t>2022.0</t>
+        </is>
       </c>
       <c r="H636" t="inlineStr">
         <is>
@@ -35188,8 +35230,10 @@
         </is>
       </c>
       <c r="F637" t="inlineStr"/>
-      <c r="G637" t="n">
-        <v>2026</v>
+      <c r="G637" t="inlineStr">
+        <is>
+          <t>2026.0</t>
+        </is>
       </c>
       <c r="H637" t="inlineStr">
         <is>
@@ -35240,8 +35284,10 @@
           <t>https://shop.flugschule-hochries.de/AIRDESIGN-Volt-5-M/SW10612</t>
         </is>
       </c>
-      <c r="F638" t="n">
-        <v>3000</v>
+      <c r="F638" t="inlineStr">
+        <is>
+          <t>3000.0</t>
+        </is>
       </c>
       <c r="G638" t="inlineStr"/>
       <c r="H638" t="inlineStr"/>
@@ -35285,8 +35331,10 @@
           <t>https://shop.flugschule-hochries.de/AIRDESIGN-Volt-5-S/SW10610</t>
         </is>
       </c>
-      <c r="F639" t="n">
-        <v>3650</v>
+      <c r="F639" t="inlineStr">
+        <is>
+          <t>3650.0</t>
+        </is>
       </c>
       <c r="G639" t="inlineStr"/>
       <c r="H639" t="inlineStr"/>
@@ -35301,6 +35349,512 @@
       <c r="M639" t="inlineStr">
         <is>
           <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="640">
+      <c r="A640" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B640" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C640" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D640" t="inlineStr">
+        <is>
+          <t>Křídlo EN B UP Summit XC 4 M 95-115kg Listovaný TK platná Křídlo EN B UP Summit XC 4 M 95-115kg Listovaný TK platná Nabí</t>
+        </is>
+      </c>
+      <c r="E640" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/up-summit-xc-4-m-95-115kg-concertinas-tc-valid-7828/</t>
+        </is>
+      </c>
+      <c r="F640" t="inlineStr"/>
+      <c r="G640" t="n">
+        <v>2021</v>
+      </c>
+      <c r="H640" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I640" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J640" t="inlineStr"/>
+      <c r="K640" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L640" t="inlineStr"/>
+      <c r="M640" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="641">
+      <c r="A641" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B641" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C641" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D641" t="inlineStr">
+        <is>
+          <t>Křídlo EN B UP KIBO X M 90-115kg Křídlo EN B UP KIBO X M 90-115kg 60 000,00 CZK EN B Velikost: M Vzletová hmotnost: 90 -</t>
+        </is>
+      </c>
+      <c r="E641" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/up-kibo-x-m-90-115kg-7824/</t>
+        </is>
+      </c>
+      <c r="F641" t="inlineStr"/>
+      <c r="G641" t="inlineStr"/>
+      <c r="H641" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I641" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J641" t="inlineStr"/>
+      <c r="K641" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L641" t="inlineStr"/>
+      <c r="M641" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="642">
+      <c r="A642" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B642" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C642" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D642" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AXIS Pluto 2 M 80-105kg Křídlo EN B AXIS Pluto 2 M 80-105kg 4 000,00 CZK EN B Velikost: M Vzletová hmotnost:</t>
+        </is>
+      </c>
+      <c r="E642" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-pluto-2-m-80-105kg-7822/</t>
+        </is>
+      </c>
+      <c r="F642" t="inlineStr"/>
+      <c r="G642" t="n">
+        <v>2014</v>
+      </c>
+      <c r="H642" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I642" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J642" t="inlineStr"/>
+      <c r="K642" t="inlineStr">
+        <is>
+          <t>Více létané (200-300h)</t>
+        </is>
+      </c>
+      <c r="L642" t="inlineStr"/>
+      <c r="M642" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="643">
+      <c r="A643" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B643" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C643" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D643" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Ozone Rush 5 L 85-105kg Listovaný Nelétáno na písku Nekoupáno Drobné opravy TK platná Křídlo EN B Ozone Rush</t>
+        </is>
+      </c>
+      <c r="E643" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/ozone-rush-5-l-85-105kg-concertinas-no-flying-on-the-san-7815/</t>
+        </is>
+      </c>
+      <c r="F643" t="inlineStr"/>
+      <c r="G643" t="n">
+        <v>2019</v>
+      </c>
+      <c r="H643" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I643" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J643" t="inlineStr"/>
+      <c r="K643" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L643" t="inlineStr"/>
+      <c r="M643" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="644">
+      <c r="A644" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B644" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C644" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D644" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AXIS Comet 3 M Listovaný Nové Žádné SIV Křídlo EN B AXIS Comet 3 M Listovaný Nové Žádné SIV 21 865,36 CZK (9</t>
+        </is>
+      </c>
+      <c r="E644" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-concertinas-new-no-sivs-7529/</t>
+        </is>
+      </c>
+      <c r="F644" t="n">
+        <v>900</v>
+      </c>
+      <c r="G644" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H644" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I644" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J644" t="inlineStr"/>
+      <c r="K644" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L644" t="inlineStr"/>
+      <c r="M644" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="645">
+      <c r="A645" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B645" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C645" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D645" t="inlineStr">
+        <is>
+          <t>Křídlo EN A UP Dena M 85-110kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá TK platná Křídlo EN A UP Dena</t>
+        </is>
+      </c>
+      <c r="E645" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/up-dena-m-85-110kg-no-sivs-no-flying-on-the-sand-no-tree-7839/</t>
+        </is>
+      </c>
+      <c r="F645" t="inlineStr"/>
+      <c r="G645" t="n">
+        <v>2022</v>
+      </c>
+      <c r="H645" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I645" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J645" t="inlineStr"/>
+      <c r="K645" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L645" t="inlineStr"/>
+      <c r="M645" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="646">
+      <c r="A646" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B646" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C646" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D646" t="inlineStr">
+        <is>
+          <t>Křídlo EN A GIN Bolero 5 m 85-105kg Drobné opravy TK platná Křídlo EN A GIN Bolero 5 m 85-105kg Drobné opravy TK platná</t>
+        </is>
+      </c>
+      <c r="E646" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/gin-bolero-5-m-85-105kg-small-repairs-tc-valid-7814/</t>
+        </is>
+      </c>
+      <c r="F646" t="inlineStr"/>
+      <c r="G646" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H646" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I646" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="J646" t="inlineStr"/>
+      <c r="K646" t="inlineStr">
+        <is>
+          <t>Olétané (více než 300h)</t>
+        </is>
+      </c>
+      <c r="L646" t="inlineStr"/>
+      <c r="M646" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="647">
+      <c r="A647" t="inlineStr">
+        <is>
+          <t>hochries_de</t>
+        </is>
+      </c>
+      <c r="B647" t="inlineStr">
+        <is>
+          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
+        </is>
+      </c>
+      <c r="C647" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D647" t="inlineStr">
+        <is>
+          <t>ADVANCE Sigma DLS 20</t>
+        </is>
+      </c>
+      <c r="E647" t="inlineStr">
+        <is>
+          <t>https://shop.flugschule-hochries.de/ADVANCE-Sigma-DLS-20/SW10843</t>
+        </is>
+      </c>
+      <c r="F647" t="n">
+        <v>3875</v>
+      </c>
+      <c r="G647" t="inlineStr"/>
+      <c r="H647" t="inlineStr"/>
+      <c r="I647" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="J647" t="inlineStr"/>
+      <c r="K647" t="inlineStr"/>
+      <c r="L647" t="inlineStr"/>
+      <c r="M647" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="648">
+      <c r="A648" t="inlineStr">
+        <is>
+          <t>hochries_de</t>
+        </is>
+      </c>
+      <c r="B648" t="inlineStr">
+        <is>
+          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
+        </is>
+      </c>
+      <c r="C648" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D648" t="inlineStr">
+        <is>
+          <t>ADVANCE Theta ULS 21</t>
+        </is>
+      </c>
+      <c r="E648" t="inlineStr">
+        <is>
+          <t>https://shop.flugschule-hochries.de/ADVANCE-Theta-ULS-21</t>
+        </is>
+      </c>
+      <c r="F648" t="n">
+        <v>3275</v>
+      </c>
+      <c r="G648" t="inlineStr"/>
+      <c r="H648" t="inlineStr"/>
+      <c r="I648" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="J648" t="inlineStr"/>
+      <c r="K648" t="inlineStr"/>
+      <c r="L648" t="inlineStr"/>
+      <c r="M648" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="649">
+      <c r="A649" t="inlineStr">
+        <is>
+          <t>hochries_de</t>
+        </is>
+      </c>
+      <c r="B649" t="inlineStr">
+        <is>
+          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
+        </is>
+      </c>
+      <c r="C649" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D649" t="inlineStr">
+        <is>
+          <t>ADVANCE Xi 23</t>
+        </is>
+      </c>
+      <c r="E649" t="inlineStr">
+        <is>
+          <t>https://shop.flugschule-hochries.de/ADVANCE-Xi-23</t>
+        </is>
+      </c>
+      <c r="F649" t="n">
+        <v>975</v>
+      </c>
+      <c r="G649" t="inlineStr"/>
+      <c r="H649" t="inlineStr"/>
+      <c r="I649" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="J649" t="inlineStr"/>
+      <c r="K649" t="inlineStr"/>
+      <c r="L649" t="inlineStr"/>
+      <c r="M649" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
         </is>
       </c>
     </row>
@@ -35315,7 +35869,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M53"/>
+  <dimension ref="A1:M63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -37280,11 +37834,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/777-rook-3-s-70-85kg-tc-valid-7800/</t>
         </is>
       </c>
-      <c r="F36" t="n">
-        <v>650</v>
-      </c>
-      <c r="G36" t="n">
-        <v>2020</v>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>650.0</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>2020.0</t>
+        </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
@@ -37335,11 +37893,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/airdesign-susi-3-21-60-108kg-no-sivs-no-flying-on-the-sa-7799/</t>
         </is>
       </c>
-      <c r="F37" t="n">
-        <v>1500</v>
-      </c>
-      <c r="G37" t="n">
-        <v>2021</v>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>1500.0</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>2021.0</t>
+        </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
@@ -37391,8 +37953,10 @@
         </is>
       </c>
       <c r="F38" t="inlineStr"/>
-      <c r="G38" t="n">
-        <v>2018</v>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>2018.0</t>
+        </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
@@ -37444,8 +38008,10 @@
         </is>
       </c>
       <c r="F39" t="inlineStr"/>
-      <c r="G39" t="n">
-        <v>2013</v>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>2013.0</t>
+        </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
@@ -37497,8 +38063,10 @@
         </is>
       </c>
       <c r="F40" t="inlineStr"/>
-      <c r="G40" t="n">
-        <v>2019</v>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>2019.0</t>
+        </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
@@ -37550,8 +38118,10 @@
         </is>
       </c>
       <c r="F41" t="inlineStr"/>
-      <c r="G41" t="n">
-        <v>2024</v>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>2024.0</t>
+        </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
@@ -37603,8 +38173,10 @@
         </is>
       </c>
       <c r="F42" t="inlineStr"/>
-      <c r="G42" t="n">
-        <v>2016</v>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>2016.0</t>
+        </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
@@ -37656,8 +38228,10 @@
         </is>
       </c>
       <c r="F43" t="inlineStr"/>
-      <c r="G43" t="n">
-        <v>2023</v>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>2023.0</t>
+        </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
@@ -37709,8 +38283,10 @@
         </is>
       </c>
       <c r="F44" t="inlineStr"/>
-      <c r="G44" t="n">
-        <v>2026</v>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>2026.0</t>
+        </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
@@ -37757,11 +38333,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/sky-paragliders-kudos-2-l-85-110kg-concertinas-no-sivs-n-7756/</t>
         </is>
       </c>
-      <c r="F45" t="n">
-        <v>2900</v>
-      </c>
-      <c r="G45" t="n">
-        <v>2025</v>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>2900.0</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>2025.0</t>
+        </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
@@ -37812,11 +38392,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-concertinas-new-no-sivs-7529/</t>
         </is>
       </c>
-      <c r="F46" t="n">
-        <v>900</v>
-      </c>
-      <c r="G46" t="n">
-        <v>2020</v>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>900.0</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>2020.0</t>
+        </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
@@ -37867,11 +38451,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/nova-prion-5-m-90-115kg-concertinas-no-sivs-no-flying-on-7790/</t>
         </is>
       </c>
-      <c r="F47" t="n">
-        <v>1200</v>
-      </c>
-      <c r="G47" t="n">
-        <v>2022</v>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>1200.0</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>2022.0</t>
+        </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
@@ -37923,8 +38511,10 @@
         </is>
       </c>
       <c r="F48" t="inlineStr"/>
-      <c r="G48" t="n">
-        <v>2016</v>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>2016.0</t>
+        </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
@@ -37976,8 +38566,10 @@
         </is>
       </c>
       <c r="F49" t="inlineStr"/>
-      <c r="G49" t="n">
-        <v>2018</v>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>2018.0</t>
+        </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
@@ -38028,11 +38620,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/mac-lucky-4-30-105-130kg-concertinas-no-sivs-no-flying-o-7780/</t>
         </is>
       </c>
-      <c r="F50" t="n">
-        <v>1600</v>
-      </c>
-      <c r="G50" t="n">
-        <v>2022</v>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>1600.0</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>2022.0</t>
+        </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
@@ -38084,8 +38680,10 @@
         </is>
       </c>
       <c r="F51" t="inlineStr"/>
-      <c r="G51" t="n">
-        <v>2026</v>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>2026.0</t>
+        </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
@@ -38136,8 +38734,10 @@
           <t>https://shop.flugschule-hochries.de/AIRDESIGN-Volt-5-M/SW10612</t>
         </is>
       </c>
-      <c r="F52" t="n">
-        <v>3000</v>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>3000.0</t>
+        </is>
       </c>
       <c r="G52" t="inlineStr"/>
       <c r="H52" t="inlineStr"/>
@@ -38181,8 +38781,10 @@
           <t>https://shop.flugschule-hochries.de/AIRDESIGN-Volt-5-S/SW10610</t>
         </is>
       </c>
-      <c r="F53" t="n">
-        <v>3650</v>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>3650.0</t>
+        </is>
       </c>
       <c r="G53" t="inlineStr"/>
       <c r="H53" t="inlineStr"/>
@@ -38197,6 +38799,512 @@
       <c r="M53" t="inlineStr">
         <is>
           <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Křídlo EN B UP Summit XC 4 M 95-115kg Listovaný TK platná Křídlo EN B UP Summit XC 4 M 95-115kg Listovaný TK platná Nabí</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/up-summit-xc-4-m-95-115kg-concertinas-tc-valid-7828/</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr"/>
+      <c r="G54" t="n">
+        <v>2021</v>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr"/>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr"/>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Křídlo EN B UP KIBO X M 90-115kg Křídlo EN B UP KIBO X M 90-115kg 60 000,00 CZK EN B Velikost: M Vzletová hmotnost: 90 -</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/up-kibo-x-m-90-115kg-7824/</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr"/>
+      <c r="G55" t="inlineStr"/>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr"/>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr"/>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AXIS Pluto 2 M 80-105kg Křídlo EN B AXIS Pluto 2 M 80-105kg 4 000,00 CZK EN B Velikost: M Vzletová hmotnost:</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-pluto-2-m-80-105kg-7822/</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr"/>
+      <c r="G56" t="n">
+        <v>2014</v>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr"/>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>Více létané (200-300h)</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr"/>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Ozone Rush 5 L 85-105kg Listovaný Nelétáno na písku Nekoupáno Drobné opravy TK platná Křídlo EN B Ozone Rush</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/ozone-rush-5-l-85-105kg-concertinas-no-flying-on-the-san-7815/</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr"/>
+      <c r="G57" t="n">
+        <v>2019</v>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr"/>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr"/>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AXIS Comet 3 M Listovaný Nové Žádné SIV Křídlo EN B AXIS Comet 3 M Listovaný Nové Žádné SIV 21 865,36 CZK (9</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-concertinas-new-no-sivs-7529/</t>
+        </is>
+      </c>
+      <c r="F58" t="n">
+        <v>900</v>
+      </c>
+      <c r="G58" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr"/>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr"/>
+      <c r="M58" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Křídlo EN A UP Dena M 85-110kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá TK platná Křídlo EN A UP Dena</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/up-dena-m-85-110kg-no-sivs-no-flying-on-the-sand-no-tree-7839/</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr"/>
+      <c r="G59" t="n">
+        <v>2022</v>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr"/>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr"/>
+      <c r="M59" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Křídlo EN A GIN Bolero 5 m 85-105kg Drobné opravy TK platná Křídlo EN A GIN Bolero 5 m 85-105kg Drobné opravy TK platná</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/gin-bolero-5-m-85-105kg-small-repairs-tc-valid-7814/</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr"/>
+      <c r="G60" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr"/>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>Olétané (více než 300h)</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr"/>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>hochries_de</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>ADVANCE Sigma DLS 20</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>https://shop.flugschule-hochries.de/ADVANCE-Sigma-DLS-20/SW10843</t>
+        </is>
+      </c>
+      <c r="F61" t="n">
+        <v>3875</v>
+      </c>
+      <c r="G61" t="inlineStr"/>
+      <c r="H61" t="inlineStr"/>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr"/>
+      <c r="K61" t="inlineStr"/>
+      <c r="L61" t="inlineStr"/>
+      <c r="M61" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>hochries_de</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>ADVANCE Theta ULS 21</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>https://shop.flugschule-hochries.de/ADVANCE-Theta-ULS-21</t>
+        </is>
+      </c>
+      <c r="F62" t="n">
+        <v>3275</v>
+      </c>
+      <c r="G62" t="inlineStr"/>
+      <c r="H62" t="inlineStr"/>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr"/>
+      <c r="K62" t="inlineStr"/>
+      <c r="L62" t="inlineStr"/>
+      <c r="M62" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>hochries_de</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>ADVANCE Xi 23</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>https://shop.flugschule-hochries.de/ADVANCE-Xi-23</t>
+        </is>
+      </c>
+      <c r="F63" t="n">
+        <v>975</v>
+      </c>
+      <c r="G63" t="inlineStr"/>
+      <c r="H63" t="inlineStr"/>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr"/>
+      <c r="K63" t="inlineStr"/>
+      <c r="L63" t="inlineStr"/>
+      <c r="M63" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
         </is>
       </c>
     </row>
@@ -38211,7 +39319,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M19"/>
+  <dimension ref="A1:M11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -38224,7 +39332,7 @@
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="25" customWidth="1" min="11" max="11"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
@@ -38314,19 +39422,17 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN B 777 Rook 3 S 70-85kg TK platná Křídlo EN B 777 Rook 3 S 70-85kg TK platná 15 900,00 CZK (650,00 EUR) EN B Ve</t>
+          <t>Křídlo EN B UP Summit XC 4 M 95-115kg Listovaný TK platná Křídlo EN B UP Summit XC 4 M 95-115kg Listovaný TK platná Nabí</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/777-rook-3-s-70-85kg-tc-valid-7800/</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>650</v>
-      </c>
+          <t>https://paragliding-bazar.cz/cs/offering/up-summit-xc-4-m-95-115kg-concertinas-tc-valid-7828/</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
       <c r="G2" t="n">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -38335,19 +39441,19 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Více létané (200-300h)</t>
+          <t>Mírně létané (50-100h)</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-26</t>
         </is>
       </c>
     </row>
@@ -38369,20 +39475,16 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Křídlo EN B AirDesign Susi 3 21 60-108kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B AirDesign</t>
+          <t>Křídlo EN B UP KIBO X M 90-115kg Křídlo EN B UP KIBO X M 90-115kg 60 000,00 CZK EN B Velikost: M Vzletová hmotnost: 90 -</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/airdesign-susi-3-21-60-108kg-no-sivs-no-flying-on-the-sa-7799/</t>
-        </is>
-      </c>
-      <c r="F3" t="n">
-        <v>1500</v>
-      </c>
-      <c r="G3" t="n">
-        <v>2021</v>
-      </c>
+          <t>https://paragliding-bazar.cz/cs/offering/up-kibo-x-m-90-115kg-7824/</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
           <t>EN B</t>
@@ -38390,7 +39492,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>M</t>
         </is>
       </c>
       <c r="J3" t="inlineStr"/>
@@ -38402,7 +39504,7 @@
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-26</t>
         </is>
       </c>
     </row>
@@ -38424,17 +39526,17 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Křídlo EN B UP Kibo M 75-95kg Listovaný Žádné SIV Nevětveno Nekoupáno TK platná Křídlo EN B UP Kibo M 75-95kg Listovaný</t>
+          <t>Křídlo EN B AXIS Pluto 2 M 80-105kg Křídlo EN B AXIS Pluto 2 M 80-105kg 4 000,00 CZK EN B Velikost: M Vzletová hmotnost:</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/up-kibo-m-75-95kg-concertinas-no-sivs-no-trees-no-water--7798/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-pluto-2-m-80-105kg-7822/</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="n">
-        <v>2018</v>
+        <v>2014</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -38449,13 +39551,13 @@
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Létané (100-200h)</t>
+          <t>Více létané (200-300h)</t>
         </is>
       </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-26</t>
         </is>
       </c>
     </row>
@@ -38477,17 +39579,17 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Křídlo EN B Gradient Golden 4 26 85-100kg Žádné SIV Nelétáno na písku Nevětveno TK platná Křídlo EN B Gradient Golden 4</t>
+          <t>Křídlo EN B Ozone Rush 5 L 85-105kg Listovaný Nelétáno na písku Nekoupáno Drobné opravy TK platná Křídlo EN B Ozone Rush</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/gradient-golden-4-26-85-100kg-no-sivs-no-flying-on-the-s-7788/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/ozone-rush-5-l-85-105kg-concertinas-no-flying-on-the-san-7815/</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="n">
-        <v>2013</v>
+        <v>2019</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -38496,19 +39598,19 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>L</t>
         </is>
       </c>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Mírně létané (50-100h)</t>
+          <t>Létané (100-200h)</t>
         </is>
       </c>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-26</t>
         </is>
       </c>
     </row>
@@ -38530,17 +39632,19 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Křídlo EN B Skyman Crosscountry 2 M 80-105kg Křídlo EN B Skyman Crosscountry 2 M 80-105kg 24 000,00 CZK EN B Velikost: M</t>
+          <t>Křídlo EN B AXIS Comet 3 M Listovaný Nové Žádné SIV Křídlo EN B AXIS Comet 3 M Listovaný Nové Žádné SIV 21 865,36 CZK (9</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/skyman-crosscountry-2-m-80-105kg-7776/</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr"/>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-concertinas-new-no-sivs-7529/</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>900</v>
+      </c>
       <c r="G6" t="n">
-        <v>2019</v>
+        <v>2020</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
@@ -38555,25 +39659,25 @@
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Létané (100-200h)</t>
+          <t>Jako nové (0-50h)</t>
         </is>
       </c>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-26</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_b</t>
+          <t>paragliding_bazar_cz_a</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN B</t>
+          <t>Paragliding Bazar CZ – EN A</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -38583,26 +39687,26 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Křídlo EN B SKY Paragliders Kudos 2 L 85-108kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá Křídlo EN B SK</t>
+          <t>Křídlo EN A UP Dena M 85-110kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá TK platná Křídlo EN A UP Dena</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/sky-paragliders-kudos-2-l-85-108kg-no-sivs-no-flying-on--7764/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/up-dena-m-85-110kg-no-sivs-no-flying-on-the-sand-no-tree-7839/</t>
         </is>
       </c>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="n">
-        <v>2024</v>
+        <v>2022</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>EN B</t>
+          <t>EN A</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>M</t>
         </is>
       </c>
       <c r="J7" t="inlineStr"/>
@@ -38614,19 +39718,19 @@
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-26</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_b</t>
+          <t>paragliding_bazar_cz_a</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN B</t>
+          <t>Paragliding Bazar CZ – EN A</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -38636,609 +39740,173 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Křídlo EN B AXIS Pluto 3 ML 95-115kg Křídlo EN B AXIS Pluto 3 ML 95-115kg 7 500,00 CZK EN B Velikost: ML Vzletová hmotno</t>
+          <t>Křídlo EN A GIN Bolero 5 m 85-105kg Drobné opravy TK platná Křídlo EN A GIN Bolero 5 m 85-105kg Drobné opravy TK platná</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/axis-pluto-3-ml-95-115kg-7763/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/gin-bolero-5-m-85-105kg-small-repairs-tc-valid-7814/</t>
         </is>
       </c>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="n">
-        <v>2016</v>
+        <v>2015</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>EN B</t>
+          <t>EN A</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>m</t>
         </is>
       </c>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Mírně létané (50-100h)</t>
+          <t>Olétané (více než 300h)</t>
         </is>
       </c>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-26</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_b</t>
+          <t>hochries_de</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN B</t>
+          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>CZ</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Křídlo EN B UP SUMMIT X M 85-110kg Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B UP SUMMIT X M 85-110kg Ne</t>
+          <t>ADVANCE Sigma DLS 20</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/up-summit-x-m-85-110kg-no-flying-on-the-sand-no-trees-no-7762/</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="n">
-        <v>2023</v>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
+          <t>https://shop.flugschule-hochries.de/ADVANCE-Sigma-DLS-20/SW10843</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>3875</v>
+      </c>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
+      <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-26</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_b</t>
+          <t>hochries_de</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN B</t>
+          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>CZ</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Křídlo EN B MAC Eden8 100-130kg Listovaný Žádné SIV Nelétáno na písku Nevětveno TK platná Křídlo EN B MAC Eden8 100-130k</t>
+          <t>ADVANCE Theta ULS 21</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/mac-eden8-100-130kg-concertinas-no-sivs-no-flying-on-the-7761/</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="n">
-        <v>2026</v>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr"/>
+          <t>https://shop.flugschule-hochries.de/ADVANCE-Theta-ULS-21</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>3275</v>
+      </c>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
       <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
+      <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-26</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_b</t>
+          <t>hochries_de</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN B</t>
+          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>CZ</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Křídlo EN B SKY Paragliders Kudos 2 L 85-110kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Křídlo EN B SKY</t>
+          <t>ADVANCE Xi 23</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/sky-paragliders-kudos-2-l-85-110kg-concertinas-no-sivs-n-7756/</t>
+          <t>https://shop.flugschule-hochries.de/ADVANCE-Xi-23</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>2900</v>
-      </c>
-      <c r="G11" t="n">
-        <v>2025</v>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
+        <v>975</v>
+      </c>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>23</t>
         </is>
       </c>
       <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
+      <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>Křídlo EN B AXIS Comet 3 M Listovaný Nové Žádné SIV Křídlo EN B AXIS Comet 3 M Listovaný Nové Žádné SIV 21 834,06 CZK (9</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-concertinas-new-no-sivs-7529/</t>
-        </is>
-      </c>
-      <c r="F12" t="n">
-        <v>900</v>
-      </c>
-      <c r="G12" t="n">
-        <v>2020</v>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr">
-        <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Křídlo EN A Nova Prion 5 M 90-115kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN A Nova</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/nova-prion-5-m-90-115kg-concertinas-no-sivs-no-flying-on-7790/</t>
-        </is>
-      </c>
-      <c r="F13" t="n">
-        <v>1200</v>
-      </c>
-      <c r="G13" t="n">
-        <v>2022</v>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Křídlo EN A MAC Lucky 4 28 85-110kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Drobné opravy TK platná Křídlo EN A</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/mac-lucky-4-28-85-110kg-no-sivs-no-flying-on-the-sand-no-7789/</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="n">
-        <v>2016</v>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>28</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>Mírně létané (50-100h)</t>
-        </is>
-      </c>
-      <c r="L14" t="inlineStr"/>
-      <c r="M14" t="inlineStr">
-        <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Křídlo EN A Gradient Bright 5 26 75-100kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá Křídlo EN A Gradien</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/gradient-bright-5-26-75-100kg-no-sivs-no-flying-on-the-s-7787/</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="n">
-        <v>2018</v>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>26</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L15" t="inlineStr"/>
-      <c r="M15" t="inlineStr">
-        <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Křídlo EN A MAC Lucky 4 30 105-130kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá (Součást kompl</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/mac-lucky-4-30-105-130kg-concertinas-no-sivs-no-flying-o-7780/</t>
-        </is>
-      </c>
-      <c r="F16" t="n">
-        <v>1600</v>
-      </c>
-      <c r="G16" t="n">
-        <v>2022</v>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>Létané (100-200h)</t>
-        </is>
-      </c>
-      <c r="L16" t="inlineStr"/>
-      <c r="M16" t="inlineStr">
-        <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>Křídlo EN A SKY Paragliders Gaia3M M 73-97kg Listovaný Nové Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Křídlo EN A</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/sky-paragliders-gaia3m-m-73-97kg-concertinas-new-no-sivs-7769/</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="n">
-        <v>2026</v>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L17" t="inlineStr"/>
-      <c r="M17" t="inlineStr">
-        <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>hochries_de</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>AIRDESIGN Volt 5 M</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>https://shop.flugschule-hochries.de/AIRDESIGN-Volt-5-M/SW10612</t>
-        </is>
-      </c>
-      <c r="F18" t="n">
-        <v>3000</v>
-      </c>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
-      <c r="L18" t="inlineStr"/>
-      <c r="M18" t="inlineStr">
-        <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>hochries_de</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>AIRDESIGN Volt 5 S</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>https://shop.flugschule-hochries.de/AIRDESIGN-Volt-5-S/SW10610</t>
-        </is>
-      </c>
-      <c r="F19" t="n">
-        <v>3650</v>
-      </c>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
-      <c r="L19" t="inlineStr"/>
-      <c r="M19" t="inlineStr">
-        <is>
-          <t>2026-09-19</t>
+          <t>2026-09-26</t>
         </is>
       </c>
     </row>
@@ -39253,7 +39921,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M5"/>
+  <dimension ref="A1:M4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -39266,7 +39934,7 @@
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="25" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
@@ -39356,16 +40024,16 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN B 777 Rook 3 S 70-85kg TK platná Křídlo EN B 777 Rook 3 S 70-85kg TK platná 15 900,00 CZK (650,00 EUR) EN B Ve</t>
+          <t>Křídlo EN B AXIS Comet 3 M Listovaný Nové Žádné SIV Křídlo EN B AXIS Comet 3 M Listovaný Nové Žádné SIV 21 865,36 CZK (9</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/777-rook-3-s-70-85kg-tc-valid-7800/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-concertinas-new-no-sivs-7529/</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>650</v>
+        <v>900</v>
       </c>
       <c r="G2" t="n">
         <v>2020</v>
@@ -39377,174 +40045,109 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Více létané (200-300h)</t>
+          <t>Jako nové (0-50h)</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-26</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_b</t>
+          <t>hochries_de</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN B</t>
+          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>CZ</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Křídlo EN B AirDesign Susi 3 21 60-108kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B AirDesign</t>
+          <t>ADVANCE Theta ULS 21</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/airdesign-susi-3-21-60-108kg-no-sivs-no-flying-on-the-sa-7799/</t>
+          <t>https://shop.flugschule-hochries.de/ADVANCE-Theta-ULS-21</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>1500</v>
-      </c>
-      <c r="G3" t="n">
-        <v>2021</v>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
+        <v>3275</v>
+      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr">
         <is>
           <t>21</t>
         </is>
       </c>
       <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
+      <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-26</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_b</t>
+          <t>hochries_de</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN B</t>
+          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>CZ</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Křídlo EN B AXIS Comet 3 M Listovaný Nové Žádné SIV Křídlo EN B AXIS Comet 3 M Listovaný Nové Žádné SIV 21 834,06 CZK (9</t>
+          <t>ADVANCE Xi 23</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-concertinas-new-no-sivs-7529/</t>
+          <t>https://shop.flugschule-hochries.de/ADVANCE-Xi-23</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>900</v>
-      </c>
-      <c r="G4" t="n">
-        <v>2020</v>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
+        <v>975</v>
+      </c>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>23</t>
         </is>
       </c>
       <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
+      <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>hochries_de</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>AIRDESIGN Volt 5 S</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>https://shop.flugschule-hochries.de/AIRDESIGN-Volt-5-S/SW10610</t>
-        </is>
-      </c>
-      <c r="F5" t="n">
-        <v>3650</v>
-      </c>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>2026-09-19</t>
+          <t>2026-09-26</t>
         </is>
       </c>
     </row>
@@ -39562,17 +40165,17 @@
   <dimension ref="A1:M2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="52" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="7" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="25" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
@@ -39647,55 +40250,45 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_b</t>
+          <t>hochries_de</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN B</t>
+          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>CZ</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN B 777 Rook 3 S 70-85kg TK platná Křídlo EN B 777 Rook 3 S 70-85kg TK platná 15 900,00 CZK (650,00 EUR) EN B Ve</t>
+          <t>ADVANCE Xi 23</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/777-rook-3-s-70-85kg-tc-valid-7800/</t>
+          <t>https://shop.flugschule-hochries.de/ADVANCE-Xi-23</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>650</v>
-      </c>
-      <c r="G2" t="n">
-        <v>2020</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
+        <v>975</v>
+      </c>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>23</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Více létané (200-300h)</t>
-        </is>
-      </c>
+      <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-26</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: bazar_watcher data update 2026-10-03
</commit_message>
<xml_diff>
--- a/data/bazar_watcher/listings.xlsx
+++ b/data/bazar_watcher/listings.xlsx
@@ -8,7 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vsechny inzeraty" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09-2026" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10-2026" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dnes pridane" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Klárka – EN A - low-B, XXS-XS" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Michal – low-B, S, do 1300 €" sheetId="5" state="visible" r:id="rId5"/>
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M649"/>
+  <dimension ref="A1:M656"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -35379,8 +35379,10 @@
         </is>
       </c>
       <c r="F640" t="inlineStr"/>
-      <c r="G640" t="n">
-        <v>2021</v>
+      <c r="G640" t="inlineStr">
+        <is>
+          <t>2021.0</t>
+        </is>
       </c>
       <c r="H640" t="inlineStr">
         <is>
@@ -35483,8 +35485,10 @@
         </is>
       </c>
       <c r="F642" t="inlineStr"/>
-      <c r="G642" t="n">
-        <v>2014</v>
+      <c r="G642" t="inlineStr">
+        <is>
+          <t>2014.0</t>
+        </is>
       </c>
       <c r="H642" t="inlineStr">
         <is>
@@ -35536,8 +35540,10 @@
         </is>
       </c>
       <c r="F643" t="inlineStr"/>
-      <c r="G643" t="n">
-        <v>2019</v>
+      <c r="G643" t="inlineStr">
+        <is>
+          <t>2019.0</t>
+        </is>
       </c>
       <c r="H643" t="inlineStr">
         <is>
@@ -35588,11 +35594,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-concertinas-new-no-sivs-7529/</t>
         </is>
       </c>
-      <c r="F644" t="n">
-        <v>900</v>
-      </c>
-      <c r="G644" t="n">
-        <v>2020</v>
+      <c r="F644" t="inlineStr">
+        <is>
+          <t>900.0</t>
+        </is>
+      </c>
+      <c r="G644" t="inlineStr">
+        <is>
+          <t>2020.0</t>
+        </is>
       </c>
       <c r="H644" t="inlineStr">
         <is>
@@ -35644,8 +35654,10 @@
         </is>
       </c>
       <c r="F645" t="inlineStr"/>
-      <c r="G645" t="n">
-        <v>2022</v>
+      <c r="G645" t="inlineStr">
+        <is>
+          <t>2022.0</t>
+        </is>
       </c>
       <c r="H645" t="inlineStr">
         <is>
@@ -35697,8 +35709,10 @@
         </is>
       </c>
       <c r="F646" t="inlineStr"/>
-      <c r="G646" t="n">
-        <v>2015</v>
+      <c r="G646" t="inlineStr">
+        <is>
+          <t>2015.0</t>
+        </is>
       </c>
       <c r="H646" t="inlineStr">
         <is>
@@ -35749,8 +35763,10 @@
           <t>https://shop.flugschule-hochries.de/ADVANCE-Sigma-DLS-20/SW10843</t>
         </is>
       </c>
-      <c r="F647" t="n">
-        <v>3875</v>
+      <c r="F647" t="inlineStr">
+        <is>
+          <t>3875.0</t>
+        </is>
       </c>
       <c r="G647" t="inlineStr"/>
       <c r="H647" t="inlineStr"/>
@@ -35794,8 +35810,10 @@
           <t>https://shop.flugschule-hochries.de/ADVANCE-Theta-ULS-21</t>
         </is>
       </c>
-      <c r="F648" t="n">
-        <v>3275</v>
+      <c r="F648" t="inlineStr">
+        <is>
+          <t>3275.0</t>
+        </is>
       </c>
       <c r="G648" t="inlineStr"/>
       <c r="H648" t="inlineStr"/>
@@ -35839,8 +35857,10 @@
           <t>https://shop.flugschule-hochries.de/ADVANCE-Xi-23</t>
         </is>
       </c>
-      <c r="F649" t="n">
-        <v>975</v>
+      <c r="F649" t="inlineStr">
+        <is>
+          <t>975.0</t>
+        </is>
       </c>
       <c r="G649" t="inlineStr"/>
       <c r="H649" t="inlineStr"/>
@@ -35855,6 +35875,373 @@
       <c r="M649" t="inlineStr">
         <is>
           <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="650">
+      <c r="A650" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B650" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C650" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D650" t="inlineStr">
+        <is>
+          <t>Křídlo EN B MAC Illusion 24 70-90kg Nelétáno na písku Nevětveno Nekoupáno TK čerstvá S listovacím obalem Křídlo EN B MAC</t>
+        </is>
+      </c>
+      <c r="E650" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/mac-illusion-24-70-90kg-no-flying-on-the-sand-no-trees-n-7863/</t>
+        </is>
+      </c>
+      <c r="F650" t="inlineStr"/>
+      <c r="G650" t="n">
+        <v>2019</v>
+      </c>
+      <c r="H650" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I650" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="J650" t="inlineStr"/>
+      <c r="K650" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L650" t="inlineStr"/>
+      <c r="M650" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="651">
+      <c r="A651" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B651" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C651" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D651" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AXIS Pluto 3 ML 90-115kg Listovaný Žádné SIV Nevětveno Drobné opravy TK platná Křídlo EN B AXIS Pluto 3 ML 9</t>
+        </is>
+      </c>
+      <c r="E651" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-pluto-3-ml-90-115kg-concertinas-no-sivs-no-trees-sm-7858/</t>
+        </is>
+      </c>
+      <c r="F651" t="inlineStr"/>
+      <c r="G651" t="n">
+        <v>2021</v>
+      </c>
+      <c r="H651" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I651" t="inlineStr">
+        <is>
+          <t>ML</t>
+        </is>
+      </c>
+      <c r="J651" t="inlineStr"/>
+      <c r="K651" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L651" t="inlineStr"/>
+      <c r="M651" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="652">
+      <c r="A652" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B652" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C652" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D652" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Nova Mentor 4 80-105kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B Nova Mentor 4 8</t>
+        </is>
+      </c>
+      <c r="E652" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-4-80-105kg-no-sivs-no-flying-on-the-sand-no--7854/</t>
+        </is>
+      </c>
+      <c r="F652" t="inlineStr"/>
+      <c r="G652" t="n">
+        <v>2018</v>
+      </c>
+      <c r="H652" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I652" t="inlineStr"/>
+      <c r="J652" t="inlineStr"/>
+      <c r="K652" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L652" t="inlineStr"/>
+      <c r="M652" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="653">
+      <c r="A653" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B653" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C653" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D653" t="inlineStr">
+        <is>
+          <t>Křídlo EN B SKY Paragliders Kudos 2 L 85-108kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá Křídlo EN B SK</t>
+        </is>
+      </c>
+      <c r="E653" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/sky-paragliders-kudos-2-l-85-108kg-no-sivs-no-flying-on--7852/</t>
+        </is>
+      </c>
+      <c r="F653" t="inlineStr"/>
+      <c r="G653" t="n">
+        <v>2024</v>
+      </c>
+      <c r="H653" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I653" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J653" t="inlineStr"/>
+      <c r="K653" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L653" t="inlineStr"/>
+      <c r="M653" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="654">
+      <c r="A654" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B654" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C654" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D654" t="inlineStr">
+        <is>
+          <t>Křídlo EN B SKY Paragliders Kudos 2 M 74-94kg Listovaný Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B SKY</t>
+        </is>
+      </c>
+      <c r="E654" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/sky-paragliders-kudos-2-m-74-94kg-concertinas-no-flying--7844/</t>
+        </is>
+      </c>
+      <c r="F654" t="inlineStr"/>
+      <c r="G654" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H654" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I654" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J654" t="inlineStr"/>
+      <c r="K654" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L654" t="inlineStr"/>
+      <c r="M654" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="655">
+      <c r="A655" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B655" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C655" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D655" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Advance Epsilon DLS 26 Křídlo EN B Advance Epsilon DLS 26 41 394,76 CZK (1 700,00 EUR) EN B Velikost: 26 Opo</t>
+        </is>
+      </c>
+      <c r="E655" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-dls-26-7734/</t>
+        </is>
+      </c>
+      <c r="F655" t="n">
+        <v>1700</v>
+      </c>
+      <c r="G655" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H655" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I655" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="J655" t="inlineStr"/>
+      <c r="K655" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L655" t="inlineStr"/>
+      <c r="M655" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="656">
+      <c r="A656" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B656" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C656" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D656" t="inlineStr">
+        <is>
+          <t>Křídlo EN A mac para Lucky 25 70-90kg Nelétáno na písku Nevětveno Nekoupáno Drobné opravy TK čerstvá Křídlo EN A mac par</t>
+        </is>
+      </c>
+      <c r="E656" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/mac-para-lucky-25-70-90kg-no-flying-on-the-sand-no-trees-7848/</t>
+        </is>
+      </c>
+      <c r="F656" t="n">
+        <v>390</v>
+      </c>
+      <c r="G656" t="n">
+        <v>2005</v>
+      </c>
+      <c r="H656" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I656" t="inlineStr"/>
+      <c r="J656" t="inlineStr"/>
+      <c r="K656" t="inlineStr">
+        <is>
+          <t>Více létané (200-300h)</t>
+        </is>
+      </c>
+      <c r="L656" t="inlineStr"/>
+      <c r="M656" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
         </is>
       </c>
     </row>
@@ -35869,20 +36256,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M63"/>
+  <dimension ref="A1:M8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="43" customWidth="1" min="11" max="11"/>
+    <col width="25" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
@@ -35972,19 +36359,17 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN B SKY Paragliders Kudos 2 M 74-94kg Nové Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Křídlo EN B SKY Parag</t>
+          <t>Křídlo EN B MAC Illusion 24 70-90kg Nelétáno na písku Nevětveno Nekoupáno TK čerstvá S listovacím obalem Křídlo EN B MAC</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/sky-paragliders-kudos-2-m-74-94kg-new-no-sivs-no-flying--7660/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/mac-illusion-24-70-90kg-no-flying-on-the-sand-no-trees-n-7863/</t>
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
+      <c r="G2" t="n">
+        <v>2019</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -35993,19 +36378,19 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>24</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Jako nové (0-50h)</t>
+          <t>Létané (100-200h)</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-10-03</t>
         </is>
       </c>
     </row>
@@ -36027,19 +36412,17 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Křídlo EN B Gradient Golden 5 26 85-105kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Křídlo EN B Gradient</t>
+          <t>Křídlo EN B AXIS Pluto 3 ML 90-115kg Listovaný Žádné SIV Nevětveno Drobné opravy TK platná Křídlo EN B AXIS Pluto 3 ML 9</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/gradient-golden-5-26-85-105kg-concertinas-no-sivs-no-fly-7675/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-pluto-3-ml-90-115kg-concertinas-no-sivs-no-trees-sm-7858/</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>2020</t>
-        </is>
+      <c r="G3" t="n">
+        <v>2021</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -36048,19 +36431,19 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Jako nové (0-50h)</t>
+          <t>Mírně létané (50-100h)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-10-03</t>
         </is>
       </c>
     </row>
@@ -36082,40 +36465,34 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Křídlo EN B UP Kibo 2 M 85-110kg Křídlo EN B UP Kibo 2 M 85-110kg 41 000,00 CZK EN B Velikost: M Vzletová hmotnost: 85 -</t>
+          <t>Křídlo EN B Nova Mentor 4 80-105kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B Nova Mentor 4 8</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/up-kibo-2-m-85-110kg-7665/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-4-80-105kg-no-sivs-no-flying-on-the-sand-no--7854/</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>2022</t>
-        </is>
+      <c r="G4" t="n">
+        <v>2018</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
           <t>EN B</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
+      <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Létané (100-200h)</t>
+          <t>Jako nové (0-50h)</t>
         </is>
       </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-10-03</t>
         </is>
       </c>
     </row>
@@ -36137,23 +36514,17 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>REZERVOVÁNO: Křídlo EN B Nova ION 7 S 90-105kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná REZERVOVÁNO: Kř</t>
+          <t>Křídlo EN B SKY Paragliders Kudos 2 L 85-108kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá Křídlo EN B SK</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/nova-ion-7-s-90-105kg-no-sivs-no-flying-on-the-sand-no-t-7522/</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>2698.0</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
+          <t>https://paragliding-bazar.cz/cs/offering/sky-paragliders-kudos-2-l-85-108kg-no-sivs-no-flying-on--7852/</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="n">
+        <v>2024</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -36162,7 +36533,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>L</t>
         </is>
       </c>
       <c r="J5" t="inlineStr"/>
@@ -36174,19 +36545,19 @@
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-10-03</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_a</t>
+          <t>paragliding_bazar_cz_b</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN A</t>
+          <t>Paragliding Bazar CZ – EN B</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -36196,40 +36567,38 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Křídlo EN A SKY Paragliders Carancho L L 93-116kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN A</t>
+          <t>Křídlo EN B SKY Paragliders Kudos 2 M 74-94kg Listovaný Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B SKY</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/sky-paragliders-carancho-l-l-93-116kg-no-sivs-no-flying--7672/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/sky-paragliders-kudos-2-m-74-94kg-concertinas-no-flying--7844/</t>
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
+      <c r="G6" t="n">
+        <v>2020</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>EN A</t>
+          <t>EN B</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>M</t>
         </is>
       </c>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Jako nové (0-50h)</t>
+          <t>Mírně létané (50-100h)</t>
         </is>
       </c>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-10-03</t>
         </is>
       </c>
     </row>
@@ -36251,19 +36620,19 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Křídlo EN B SKY Paragliders Kudos 2 L 85-110kg Listovaný Nelétáno na písku Nevětveno Drobné opravy S batohe (Součást kom</t>
+          <t>Křídlo EN B Advance Epsilon DLS 26 Křídlo EN B Advance Epsilon DLS 26 41 394,76 CZK (1 700,00 EUR) EN B Velikost: 26 Opo</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/sky-paragliders-kudos-2-l-85-110kg-concertinas-no-flying-7683/</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>2004.0</t>
-        </is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-dls-26-7734/</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>1700</v>
+      </c>
+      <c r="G7" t="n">
+        <v>2023</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -36272,31 +36641,31 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>26</t>
         </is>
       </c>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Jako nové (0-50h)</t>
+          <t>Létané (100-200h)</t>
         </is>
       </c>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-10-03</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_b</t>
+          <t>paragliding_bazar_cz_a</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN B</t>
+          <t>Paragliding Bazar CZ – EN A</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -36306,3005 +36675,36 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Křídlo EN B SKY Paragliders Kudos 2 XL 99-125kg Nové Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Křídlo EN B SKY Par</t>
+          <t>Křídlo EN A mac para Lucky 25 70-90kg Nelétáno na písku Nevětveno Nekoupáno Drobné opravy TK čerstvá Křídlo EN A mac par</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/sky-paragliders-kudos-2-xl-99-125kg-new-no-sivs-no-flyin-7682/</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>2026.0</t>
-        </is>
+          <t>https://paragliding-bazar.cz/cs/offering/mac-para-lucky-25-70-90kg-no-flying-on-the-sand-no-trees-7848/</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>390</v>
+      </c>
+      <c r="G8" t="n">
+        <v>2005</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>XL</t>
-        </is>
-      </c>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Jako nové (0-50h)</t>
+          <t>Více létané (200-300h)</t>
         </is>
       </c>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Křídlo EN A GIN Bolero 5 S 75-95kg Žádné SIV Nelétáno na písku TK čerstvá TK platná (Součást kompletu) Křídlo EN A GIN B</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/gin-bolero-5-s-75-95kg-no-sivs-no-flying-on-the-sand-tc--7678/</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>2020.0</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>Létané (100-200h)</t>
-        </is>
-      </c>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>2026-09-04</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>paraglidingshop_ch</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Paraglidingshop CH – Occasionen</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>CH</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Advance Alpha 4</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>https://paraglidingshop.ch/Advance-Alpha-4/SW10820</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>476.0</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>2026-09-04</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>paraglidingshop_ch</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Paraglidingshop CH – Occasionen</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>CH</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Occasion Ozone - Mojo 4 XL</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>https://paraglidingshop.ch/Occasion-Ozone-Mojo-4-XL/SW10819</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>381.0</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>2026.0</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>XL</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>2026-09-04</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>Křídlo EN B UP Kibo 2 M 85-110kg Křídlo EN B UP Kibo 2 M 85-110kg 35 000,00 CZK EN B Velikost: M Vzletová hmotnost: 85 -</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/up-kibo-2-m-85-110kg-7665/</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>2022</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>Létané (100-200h)</t>
-        </is>
-      </c>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr">
-        <is>
-          <t>2026-09-05</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Křídlo EN B PHI Beat 75-95kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná S batohem TOP Křídlo EN</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/phi-beat-75-95kg-concertinas-no-sivs-no-flying-on-the-sa-7722/</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>2020</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t>2026-09-08</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Křídlo EN B SKY Kudos S 64-81kg Listovaný Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B SKY Kudos S 64-81k</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/sky-kudos-s-64-81kg-concertinas-no-flying-on-the-sand-no-7721/</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>2018</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>Mírně létané (50-100h)</t>
-        </is>
-      </c>
-      <c r="L14" t="inlineStr"/>
-      <c r="M14" t="inlineStr">
-        <is>
-          <t>2026-09-08</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Křídlo EN B AXIS Comet 4 L Listovaný Žádné SIV Nelétáno na písku Nekoupáno TK čerstvá TK platná Křídlo EN B AXIS Comet 4</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-4-l-concertinas-no-sivs-no-flying-on-the-sand-7706/</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>2024</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L15" t="inlineStr"/>
-      <c r="M15" t="inlineStr">
-        <is>
-          <t>2026-09-08</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Křídlo EN B SKY Kudos S 64-81kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B SKY Kudo</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/sky-kudos-s-64-81kg-concertinas-no-sivs-no-flying-on-the-7721/</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>2018</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>Mírně létané (50-100h)</t>
-        </is>
-      </c>
-      <c r="L16" t="inlineStr"/>
-      <c r="M16" t="inlineStr">
-        <is>
-          <t>2026-09-09</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>Křídlo EN A UP MANA Listovaný Odlehčeno Nevětveno Nekoupáno TK platná Křídlo EN A UP MANA Listovaný Odlehčeno Nevětveno</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/up-mana-concertinas-lightened-no-trees-no-water-tc-valid-7731/</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>2022</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L17" t="inlineStr"/>
-      <c r="M17" t="inlineStr">
-        <is>
-          <t>2026-09-09</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>Křídlo EN B UP Kibo 2 M 85-110kg Křídlo EN B UP Kibo 2 M 85-110kg 35 000,00 CZK EN B Velikost: M Vzletová hmotnost: 85 -</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/up-kibo-2-m-85-110kg-7737/</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>2022.0</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>Létané (100-200h)</t>
-        </is>
-      </c>
-      <c r="L18" t="inlineStr"/>
-      <c r="M18" t="inlineStr">
-        <is>
-          <t>2026-09-10</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>Křídlo EN B Advance Epsilon DLS 26 Křídlo EN B Advance Epsilon DLS 26 41 071,73 CZK (1 700,00 EUR) EN B Velikost: 26 Opo</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-dls-26-7734/</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>1700.0</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>2023.0</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>26</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>Létané (100-200h)</t>
-        </is>
-      </c>
-      <c r="L19" t="inlineStr"/>
-      <c r="M19" t="inlineStr">
-        <is>
-          <t>2026-09-10</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>Křídlo EN A Advance Alpha 7 24 60-95kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN A A</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-7-24-60-95kg-concertinas-no-sivs-no-flying-7735/</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>2022.0</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>24</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>Mírně létané (50-100h)</t>
-        </is>
-      </c>
-      <c r="L20" t="inlineStr"/>
-      <c r="M20" t="inlineStr">
-        <is>
-          <t>2026-09-10</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>Křídlo EN A Advance Pi 3 25 80-120kg Křídlo EN A Advance Pi 3 25 80-120kg 48 000,00 CZK EN A Velikost: 25 Vzletová hmotn</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-pi-3-25-80-120kg-7317/</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>2021.0</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>25</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>Mírně létané (50-100h)</t>
-        </is>
-      </c>
-      <c r="L21" t="inlineStr"/>
-      <c r="M21" t="inlineStr">
-        <is>
-          <t>2026-09-10</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>paraglidingshop_ch</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Paraglidingshop CH – Occasionen</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>CH</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>Advance Alpha 5 Occasion</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>https://paraglidingshop.ch/Advance-Alpha-5-Occasion/SW10822</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>714.0</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
-      <c r="L22" t="inlineStr"/>
-      <c r="M22" t="inlineStr">
-        <is>
-          <t>2026-09-10</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>paraglidingshop_ch</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Paraglidingshop CH – Occasionen</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>CH</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>Advance Iota 26  Occasion</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>https://paraglidingshop.ch/Advance-Iota-26-Occasion/SW10821</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>905.0</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr"/>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>26</t>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr"/>
-      <c r="L23" t="inlineStr"/>
-      <c r="M23" t="inlineStr">
-        <is>
-          <t>2026-09-10</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>Křídlo EN A Drift carancho M 80-103kg Listovaný Nové Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TOP Křídlo EN A Dri</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/drift-carancho-m-80-103kg-concertinas-new-no-sivs-no-fly-7341/</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>2024</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L24" t="inlineStr"/>
-      <c r="M24" t="inlineStr">
-        <is>
-          <t>2026-09-11</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>Křídlo EN A MAC Muse 5 29 85-110kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá TOP Křídlo EN A</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/mac-muse-5-29-85-110kg-concertinas-no-sivs-no-flying-on--7732/</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>1300.0</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>2022</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>29</t>
-        </is>
-      </c>
-      <c r="J25" t="inlineStr"/>
-      <c r="K25" t="inlineStr">
-        <is>
-          <t>Mírně létané (50-100h)</t>
-        </is>
-      </c>
-      <c r="L25" t="inlineStr"/>
-      <c r="M25" t="inlineStr">
-        <is>
-          <t>2026-09-11</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>paragliding_store_at</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Paragliding Store AT – Used</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>Advance PI 3 21 fire</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>https://www.paragliding-store.at/shop/gebrauchtmarkt-used-stuff/used-paragliders/</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>1780.0</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>2022</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr"/>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>21</t>
-        </is>
-      </c>
-      <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr">
-        <is>
-          <t>sehr guter Zustand --&gt; neuer Check siehe</t>
-        </is>
-      </c>
-      <c r="L26" t="inlineStr"/>
-      <c r="M26" t="inlineStr">
-        <is>
-          <t>2026-09-11</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>Křídlo EN B Advance Epsilon DLS 26 Křídlo EN B Advance Epsilon DLS 26 41 242,12 CZK (1 700,00 EUR) EN B Velikost: 26 Opo</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-dls-26-7734/</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>1700.0</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>2023</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>26</t>
-        </is>
-      </c>
-      <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr">
-        <is>
-          <t>Létané (100-200h)</t>
-        </is>
-      </c>
-      <c r="L27" t="inlineStr"/>
-      <c r="M27" t="inlineStr">
-        <is>
-          <t>2026-09-12</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>Křídlo EN A Gradient Golden 4 24 75-100kg Listovaný Žádné SIV Nelétáno na písku Nekoupáno TK čerstvá Křídlo EN A Gradien</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/gradient-golden-4-24-75-100kg-concertinas-no-sivs-no-fly-7749/</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr"/>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>2020</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t>24</t>
-        </is>
-      </c>
-      <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L28" t="inlineStr"/>
-      <c r="M28" t="inlineStr">
-        <is>
-          <t>2026-09-12</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>Křídlo EN A Advance Alpha 6 26 70-110kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstv Křídlo EN A</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-alpha-6-26-70-110kg-concertinas-no-sivs-no-flyin-7748/</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr"/>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>2019</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I29" t="inlineStr">
-        <is>
-          <t>26</t>
-        </is>
-      </c>
-      <c r="J29" t="inlineStr"/>
-      <c r="K29" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L29" t="inlineStr"/>
-      <c r="M29" t="inlineStr">
-        <is>
-          <t>2026-09-12</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>Křídlo EN A SKY Paragliders Carancho L 93-116kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN A SK</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/sky-paragliders-carancho-l-93-116kg-no-sivs-no-flying-on-7746/</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>2005</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I30" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="J30" t="inlineStr"/>
-      <c r="K30" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L30" t="inlineStr"/>
-      <c r="M30" t="inlineStr">
-        <is>
-          <t>2026-09-12</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>Křídlo EN B Ozone Buzz z4 S 65-85kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B Ozon</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/ozone-buzz-z4-s-65-85kg-concertinas-no-sivs-no-flying-on-7753/</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr"/>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>2015</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I31" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="J31" t="inlineStr"/>
-      <c r="K31" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L31" t="inlineStr"/>
-      <c r="M31" t="inlineStr">
-        <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>Křídlo EN B Gradient Golden 4 26 85-100kg TK čerstvá TK platná S listovacím obalem Křídlo EN B Gradient Golden 4 26 85-1</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/gradient-golden-4-26-85-100kg-tc-fresh-tc-valid-with-lis-7751/</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>620.0</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>2016</t>
-        </is>
-      </c>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I32" t="inlineStr">
-        <is>
-          <t>26</t>
-        </is>
-      </c>
-      <c r="J32" t="inlineStr"/>
-      <c r="K32" t="inlineStr">
-        <is>
-          <t>Létané (100-200h)</t>
-        </is>
-      </c>
-      <c r="L32" t="inlineStr"/>
-      <c r="M32" t="inlineStr">
-        <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>Křídlo EN B Advance Epsilon DLS 26 Křídlo EN B Advance Epsilon DLS 26 41 225,11 CZK (1 700,00 EUR) EN B Velikost: 26 Opo</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-dls-26-7734/</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>1700.0</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>2023</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I33" t="inlineStr">
-        <is>
-          <t>26</t>
-        </is>
-      </c>
-      <c r="J33" t="inlineStr"/>
-      <c r="K33" t="inlineStr">
-        <is>
-          <t>Létané (100-200h)</t>
-        </is>
-      </c>
-      <c r="L33" t="inlineStr"/>
-      <c r="M33" t="inlineStr">
-        <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>Křídlo EN B MAC Eden 7 26 80-105kg TK čerstvá TK platná Křídlo EN B MAC Eden 7 26 80-105kg TK čerstvá TK platná 18 000,0</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/mac-eden-7-26-80-105kg-tc-fresh-tc-valid-7593/</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr"/>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>2022</t>
-        </is>
-      </c>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I34" t="inlineStr">
-        <is>
-          <t>26</t>
-        </is>
-      </c>
-      <c r="J34" t="inlineStr"/>
-      <c r="K34" t="inlineStr">
-        <is>
-          <t>Létané (100-200h)</t>
-        </is>
-      </c>
-      <c r="L34" t="inlineStr"/>
-      <c r="M34" t="inlineStr">
-        <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>Křídlo EN A Drift carancho S 69-90kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN A Drift caranch</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/drift-carancho-s-69-90kg-no-sivs-no-flying-on-the-sand-n-7752/</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>1800.0</t>
-        </is>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>2024</t>
-        </is>
-      </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I35" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="J35" t="inlineStr"/>
-      <c r="K35" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L35" t="inlineStr"/>
-      <c r="M35" t="inlineStr">
-        <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>Křídlo EN B 777 Rook 3 S 70-85kg TK platná Křídlo EN B 777 Rook 3 S 70-85kg TK platná 15 900,00 CZK (650,00 EUR) EN B Ve</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/777-rook-3-s-70-85kg-tc-valid-7800/</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>650.0</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>2020.0</t>
-        </is>
-      </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I36" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="J36" t="inlineStr"/>
-      <c r="K36" t="inlineStr">
-        <is>
-          <t>Více létané (200-300h)</t>
-        </is>
-      </c>
-      <c r="L36" t="inlineStr"/>
-      <c r="M36" t="inlineStr">
-        <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>Křídlo EN B AirDesign Susi 3 21 60-108kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B AirDesign</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/airdesign-susi-3-21-60-108kg-no-sivs-no-flying-on-the-sa-7799/</t>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>1500.0</t>
-        </is>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>2021.0</t>
-        </is>
-      </c>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I37" t="inlineStr">
-        <is>
-          <t>21</t>
-        </is>
-      </c>
-      <c r="J37" t="inlineStr"/>
-      <c r="K37" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L37" t="inlineStr"/>
-      <c r="M37" t="inlineStr">
-        <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>Křídlo EN B UP Kibo M 75-95kg Listovaný Žádné SIV Nevětveno Nekoupáno TK platná Křídlo EN B UP Kibo M 75-95kg Listovaný</t>
-        </is>
-      </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/up-kibo-m-75-95kg-concertinas-no-sivs-no-trees-no-water--7798/</t>
-        </is>
-      </c>
-      <c r="F38" t="inlineStr"/>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>2018.0</t>
-        </is>
-      </c>
-      <c r="H38" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I38" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J38" t="inlineStr"/>
-      <c r="K38" t="inlineStr">
-        <is>
-          <t>Létané (100-200h)</t>
-        </is>
-      </c>
-      <c r="L38" t="inlineStr"/>
-      <c r="M38" t="inlineStr">
-        <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>Křídlo EN B Gradient Golden 4 26 85-100kg Žádné SIV Nelétáno na písku Nevětveno TK platná Křídlo EN B Gradient Golden 4</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/gradient-golden-4-26-85-100kg-no-sivs-no-flying-on-the-s-7788/</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr"/>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>2013.0</t>
-        </is>
-      </c>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I39" t="inlineStr">
-        <is>
-          <t>26</t>
-        </is>
-      </c>
-      <c r="J39" t="inlineStr"/>
-      <c r="K39" t="inlineStr">
-        <is>
-          <t>Mírně létané (50-100h)</t>
-        </is>
-      </c>
-      <c r="L39" t="inlineStr"/>
-      <c r="M39" t="inlineStr">
-        <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>Křídlo EN B Skyman Crosscountry 2 M 80-105kg Křídlo EN B Skyman Crosscountry 2 M 80-105kg 24 000,00 CZK EN B Velikost: M</t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/skyman-crosscountry-2-m-80-105kg-7776/</t>
-        </is>
-      </c>
-      <c r="F40" t="inlineStr"/>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>2019.0</t>
-        </is>
-      </c>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I40" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J40" t="inlineStr"/>
-      <c r="K40" t="inlineStr">
-        <is>
-          <t>Létané (100-200h)</t>
-        </is>
-      </c>
-      <c r="L40" t="inlineStr"/>
-      <c r="M40" t="inlineStr">
-        <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>Křídlo EN B SKY Paragliders Kudos 2 L 85-108kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá Křídlo EN B SK</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/sky-paragliders-kudos-2-l-85-108kg-no-sivs-no-flying-on--7764/</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr"/>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>2024.0</t>
-        </is>
-      </c>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I41" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="J41" t="inlineStr"/>
-      <c r="K41" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L41" t="inlineStr"/>
-      <c r="M41" t="inlineStr">
-        <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>Křídlo EN B AXIS Pluto 3 ML 95-115kg Křídlo EN B AXIS Pluto 3 ML 95-115kg 7 500,00 CZK EN B Velikost: ML Vzletová hmotno</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/axis-pluto-3-ml-95-115kg-7763/</t>
-        </is>
-      </c>
-      <c r="F42" t="inlineStr"/>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t>2016.0</t>
-        </is>
-      </c>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I42" t="inlineStr">
-        <is>
-          <t>ML</t>
-        </is>
-      </c>
-      <c r="J42" t="inlineStr"/>
-      <c r="K42" t="inlineStr">
-        <is>
-          <t>Mírně létané (50-100h)</t>
-        </is>
-      </c>
-      <c r="L42" t="inlineStr"/>
-      <c r="M42" t="inlineStr">
-        <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>Křídlo EN B UP SUMMIT X M 85-110kg Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B UP SUMMIT X M 85-110kg Ne</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/up-summit-x-m-85-110kg-no-flying-on-the-sand-no-trees-no-7762/</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr"/>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>2023.0</t>
-        </is>
-      </c>
-      <c r="H43" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I43" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J43" t="inlineStr"/>
-      <c r="K43" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L43" t="inlineStr"/>
-      <c r="M43" t="inlineStr">
-        <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>Křídlo EN B MAC Eden8 100-130kg Listovaný Žádné SIV Nelétáno na písku Nevětveno TK platná Křídlo EN B MAC Eden8 100-130k</t>
-        </is>
-      </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/mac-eden8-100-130kg-concertinas-no-sivs-no-flying-on-the-7761/</t>
-        </is>
-      </c>
-      <c r="F44" t="inlineStr"/>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>2026.0</t>
-        </is>
-      </c>
-      <c r="H44" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I44" t="inlineStr"/>
-      <c r="J44" t="inlineStr"/>
-      <c r="K44" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L44" t="inlineStr"/>
-      <c r="M44" t="inlineStr">
-        <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>Křídlo EN B SKY Paragliders Kudos 2 L 85-110kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Křídlo EN B SKY</t>
-        </is>
-      </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/sky-paragliders-kudos-2-l-85-110kg-concertinas-no-sivs-n-7756/</t>
-        </is>
-      </c>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>2900.0</t>
-        </is>
-      </c>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>2025.0</t>
-        </is>
-      </c>
-      <c r="H45" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I45" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="J45" t="inlineStr"/>
-      <c r="K45" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L45" t="inlineStr"/>
-      <c r="M45" t="inlineStr">
-        <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>Křídlo EN B AXIS Comet 3 M Listovaný Nové Žádné SIV Křídlo EN B AXIS Comet 3 M Listovaný Nové Žádné SIV 21 834,06 CZK (9</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-concertinas-new-no-sivs-7529/</t>
-        </is>
-      </c>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>900.0</t>
-        </is>
-      </c>
-      <c r="G46" t="inlineStr">
-        <is>
-          <t>2020.0</t>
-        </is>
-      </c>
-      <c r="H46" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I46" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J46" t="inlineStr"/>
-      <c r="K46" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L46" t="inlineStr"/>
-      <c r="M46" t="inlineStr">
-        <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>Křídlo EN A Nova Prion 5 M 90-115kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN A Nova</t>
-        </is>
-      </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/nova-prion-5-m-90-115kg-concertinas-no-sivs-no-flying-on-7790/</t>
-        </is>
-      </c>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>1200.0</t>
-        </is>
-      </c>
-      <c r="G47" t="inlineStr">
-        <is>
-          <t>2022.0</t>
-        </is>
-      </c>
-      <c r="H47" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I47" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J47" t="inlineStr"/>
-      <c r="K47" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L47" t="inlineStr"/>
-      <c r="M47" t="inlineStr">
-        <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>Křídlo EN A MAC Lucky 4 28 85-110kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Drobné opravy TK platná Křídlo EN A</t>
-        </is>
-      </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/mac-lucky-4-28-85-110kg-no-sivs-no-flying-on-the-sand-no-7789/</t>
-        </is>
-      </c>
-      <c r="F48" t="inlineStr"/>
-      <c r="G48" t="inlineStr">
-        <is>
-          <t>2016.0</t>
-        </is>
-      </c>
-      <c r="H48" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I48" t="inlineStr">
-        <is>
-          <t>28</t>
-        </is>
-      </c>
-      <c r="J48" t="inlineStr"/>
-      <c r="K48" t="inlineStr">
-        <is>
-          <t>Mírně létané (50-100h)</t>
-        </is>
-      </c>
-      <c r="L48" t="inlineStr"/>
-      <c r="M48" t="inlineStr">
-        <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>Křídlo EN A Gradient Bright 5 26 75-100kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá Křídlo EN A Gradien</t>
-        </is>
-      </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/gradient-bright-5-26-75-100kg-no-sivs-no-flying-on-the-s-7787/</t>
-        </is>
-      </c>
-      <c r="F49" t="inlineStr"/>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t>2018.0</t>
-        </is>
-      </c>
-      <c r="H49" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I49" t="inlineStr">
-        <is>
-          <t>26</t>
-        </is>
-      </c>
-      <c r="J49" t="inlineStr"/>
-      <c r="K49" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L49" t="inlineStr"/>
-      <c r="M49" t="inlineStr">
-        <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>Křídlo EN A MAC Lucky 4 30 105-130kg Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá (Součást kompl</t>
-        </is>
-      </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/mac-lucky-4-30-105-130kg-concertinas-no-sivs-no-flying-o-7780/</t>
-        </is>
-      </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>1600.0</t>
-        </is>
-      </c>
-      <c r="G50" t="inlineStr">
-        <is>
-          <t>2022.0</t>
-        </is>
-      </c>
-      <c r="H50" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I50" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
-      </c>
-      <c r="J50" t="inlineStr"/>
-      <c r="K50" t="inlineStr">
-        <is>
-          <t>Létané (100-200h)</t>
-        </is>
-      </c>
-      <c r="L50" t="inlineStr"/>
-      <c r="M50" t="inlineStr">
-        <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>Křídlo EN A SKY Paragliders Gaia3M M 73-97kg Listovaný Nové Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Křídlo EN A</t>
-        </is>
-      </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/sky-paragliders-gaia3m-m-73-97kg-concertinas-new-no-sivs-7769/</t>
-        </is>
-      </c>
-      <c r="F51" t="inlineStr"/>
-      <c r="G51" t="inlineStr">
-        <is>
-          <t>2026.0</t>
-        </is>
-      </c>
-      <c r="H51" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I51" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J51" t="inlineStr"/>
-      <c r="K51" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L51" t="inlineStr"/>
-      <c r="M51" t="inlineStr">
-        <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>hochries_de</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>AIRDESIGN Volt 5 M</t>
-        </is>
-      </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>https://shop.flugschule-hochries.de/AIRDESIGN-Volt-5-M/SW10612</t>
-        </is>
-      </c>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t>3000.0</t>
-        </is>
-      </c>
-      <c r="G52" t="inlineStr"/>
-      <c r="H52" t="inlineStr"/>
-      <c r="I52" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J52" t="inlineStr"/>
-      <c r="K52" t="inlineStr"/>
-      <c r="L52" t="inlineStr"/>
-      <c r="M52" t="inlineStr">
-        <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>hochries_de</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>AIRDESIGN Volt 5 S</t>
-        </is>
-      </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>https://shop.flugschule-hochries.de/AIRDESIGN-Volt-5-S/SW10610</t>
-        </is>
-      </c>
-      <c r="F53" t="inlineStr">
-        <is>
-          <t>3650.0</t>
-        </is>
-      </c>
-      <c r="G53" t="inlineStr"/>
-      <c r="H53" t="inlineStr"/>
-      <c r="I53" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="J53" t="inlineStr"/>
-      <c r="K53" t="inlineStr"/>
-      <c r="L53" t="inlineStr"/>
-      <c r="M53" t="inlineStr">
-        <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>Křídlo EN B UP Summit XC 4 M 95-115kg Listovaný TK platná Křídlo EN B UP Summit XC 4 M 95-115kg Listovaný TK platná Nabí</t>
-        </is>
-      </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/up-summit-xc-4-m-95-115kg-concertinas-tc-valid-7828/</t>
-        </is>
-      </c>
-      <c r="F54" t="inlineStr"/>
-      <c r="G54" t="n">
-        <v>2021</v>
-      </c>
-      <c r="H54" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I54" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J54" t="inlineStr"/>
-      <c r="K54" t="inlineStr">
-        <is>
-          <t>Mírně létané (50-100h)</t>
-        </is>
-      </c>
-      <c r="L54" t="inlineStr"/>
-      <c r="M54" t="inlineStr">
-        <is>
-          <t>2026-09-26</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>Křídlo EN B UP KIBO X M 90-115kg Křídlo EN B UP KIBO X M 90-115kg 60 000,00 CZK EN B Velikost: M Vzletová hmotnost: 90 -</t>
-        </is>
-      </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/up-kibo-x-m-90-115kg-7824/</t>
-        </is>
-      </c>
-      <c r="F55" t="inlineStr"/>
-      <c r="G55" t="inlineStr"/>
-      <c r="H55" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I55" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J55" t="inlineStr"/>
-      <c r="K55" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L55" t="inlineStr"/>
-      <c r="M55" t="inlineStr">
-        <is>
-          <t>2026-09-26</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>Křídlo EN B AXIS Pluto 2 M 80-105kg Křídlo EN B AXIS Pluto 2 M 80-105kg 4 000,00 CZK EN B Velikost: M Vzletová hmotnost:</t>
-        </is>
-      </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/axis-pluto-2-m-80-105kg-7822/</t>
-        </is>
-      </c>
-      <c r="F56" t="inlineStr"/>
-      <c r="G56" t="n">
-        <v>2014</v>
-      </c>
-      <c r="H56" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I56" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J56" t="inlineStr"/>
-      <c r="K56" t="inlineStr">
-        <is>
-          <t>Více létané (200-300h)</t>
-        </is>
-      </c>
-      <c r="L56" t="inlineStr"/>
-      <c r="M56" t="inlineStr">
-        <is>
-          <t>2026-09-26</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>Křídlo EN B Ozone Rush 5 L 85-105kg Listovaný Nelétáno na písku Nekoupáno Drobné opravy TK platná Křídlo EN B Ozone Rush</t>
-        </is>
-      </c>
-      <c r="E57" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/ozone-rush-5-l-85-105kg-concertinas-no-flying-on-the-san-7815/</t>
-        </is>
-      </c>
-      <c r="F57" t="inlineStr"/>
-      <c r="G57" t="n">
-        <v>2019</v>
-      </c>
-      <c r="H57" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I57" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="J57" t="inlineStr"/>
-      <c r="K57" t="inlineStr">
-        <is>
-          <t>Létané (100-200h)</t>
-        </is>
-      </c>
-      <c r="L57" t="inlineStr"/>
-      <c r="M57" t="inlineStr">
-        <is>
-          <t>2026-09-26</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>Křídlo EN B AXIS Comet 3 M Listovaný Nové Žádné SIV Křídlo EN B AXIS Comet 3 M Listovaný Nové Žádné SIV 21 865,36 CZK (9</t>
-        </is>
-      </c>
-      <c r="E58" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-concertinas-new-no-sivs-7529/</t>
-        </is>
-      </c>
-      <c r="F58" t="n">
-        <v>900</v>
-      </c>
-      <c r="G58" t="n">
-        <v>2020</v>
-      </c>
-      <c r="H58" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I58" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J58" t="inlineStr"/>
-      <c r="K58" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L58" t="inlineStr"/>
-      <c r="M58" t="inlineStr">
-        <is>
-          <t>2026-09-26</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>Křídlo EN A UP Dena M 85-110kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá TK platná Křídlo EN A UP Dena</t>
-        </is>
-      </c>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/up-dena-m-85-110kg-no-sivs-no-flying-on-the-sand-no-tree-7839/</t>
-        </is>
-      </c>
-      <c r="F59" t="inlineStr"/>
-      <c r="G59" t="n">
-        <v>2022</v>
-      </c>
-      <c r="H59" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I59" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J59" t="inlineStr"/>
-      <c r="K59" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L59" t="inlineStr"/>
-      <c r="M59" t="inlineStr">
-        <is>
-          <t>2026-09-26</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_a</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN A</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D60" t="inlineStr">
-        <is>
-          <t>Křídlo EN A GIN Bolero 5 m 85-105kg Drobné opravy TK platná Křídlo EN A GIN Bolero 5 m 85-105kg Drobné opravy TK platná</t>
-        </is>
-      </c>
-      <c r="E60" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/gin-bolero-5-m-85-105kg-small-repairs-tc-valid-7814/</t>
-        </is>
-      </c>
-      <c r="F60" t="inlineStr"/>
-      <c r="G60" t="n">
-        <v>2015</v>
-      </c>
-      <c r="H60" t="inlineStr">
-        <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I60" t="inlineStr">
-        <is>
-          <t>m</t>
-        </is>
-      </c>
-      <c r="J60" t="inlineStr"/>
-      <c r="K60" t="inlineStr">
-        <is>
-          <t>Olétané (více než 300h)</t>
-        </is>
-      </c>
-      <c r="L60" t="inlineStr"/>
-      <c r="M60" t="inlineStr">
-        <is>
-          <t>2026-09-26</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>hochries_de</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
-        </is>
-      </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>ADVANCE Sigma DLS 20</t>
-        </is>
-      </c>
-      <c r="E61" t="inlineStr">
-        <is>
-          <t>https://shop.flugschule-hochries.de/ADVANCE-Sigma-DLS-20/SW10843</t>
-        </is>
-      </c>
-      <c r="F61" t="n">
-        <v>3875</v>
-      </c>
-      <c r="G61" t="inlineStr"/>
-      <c r="H61" t="inlineStr"/>
-      <c r="I61" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="J61" t="inlineStr"/>
-      <c r="K61" t="inlineStr"/>
-      <c r="L61" t="inlineStr"/>
-      <c r="M61" t="inlineStr">
-        <is>
-          <t>2026-09-26</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>hochries_de</t>
-        </is>
-      </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
-        </is>
-      </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t>ADVANCE Theta ULS 21</t>
-        </is>
-      </c>
-      <c r="E62" t="inlineStr">
-        <is>
-          <t>https://shop.flugschule-hochries.de/ADVANCE-Theta-ULS-21</t>
-        </is>
-      </c>
-      <c r="F62" t="n">
-        <v>3275</v>
-      </c>
-      <c r="G62" t="inlineStr"/>
-      <c r="H62" t="inlineStr"/>
-      <c r="I62" t="inlineStr">
-        <is>
-          <t>21</t>
-        </is>
-      </c>
-      <c r="J62" t="inlineStr"/>
-      <c r="K62" t="inlineStr"/>
-      <c r="L62" t="inlineStr"/>
-      <c r="M62" t="inlineStr">
-        <is>
-          <t>2026-09-26</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>hochries_de</t>
-        </is>
-      </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
-        </is>
-      </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>ADVANCE Xi 23</t>
-        </is>
-      </c>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t>https://shop.flugschule-hochries.de/ADVANCE-Xi-23</t>
-        </is>
-      </c>
-      <c r="F63" t="n">
-        <v>975</v>
-      </c>
-      <c r="G63" t="inlineStr"/>
-      <c r="H63" t="inlineStr"/>
-      <c r="I63" t="inlineStr">
-        <is>
-          <t>23</t>
-        </is>
-      </c>
-      <c r="J63" t="inlineStr"/>
-      <c r="K63" t="inlineStr"/>
-      <c r="L63" t="inlineStr"/>
-      <c r="M63" t="inlineStr">
-        <is>
-          <t>2026-09-26</t>
+          <t>2026-10-03</t>
         </is>
       </c>
     </row>
@@ -39319,20 +36719,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M11"/>
+  <dimension ref="A1:M8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="26" customWidth="1" min="11" max="11"/>
+    <col width="25" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
@@ -39422,17 +36822,17 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN B UP Summit XC 4 M 95-115kg Listovaný TK platná Křídlo EN B UP Summit XC 4 M 95-115kg Listovaný TK platná Nabí</t>
+          <t>Křídlo EN B MAC Illusion 24 70-90kg Nelétáno na písku Nevětveno Nekoupáno TK čerstvá S listovacím obalem Křídlo EN B MAC</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/up-summit-xc-4-m-95-115kg-concertinas-tc-valid-7828/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/mac-illusion-24-70-90kg-no-flying-on-the-sand-no-trees-n-7863/</t>
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="n">
-        <v>2021</v>
+        <v>2019</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -39441,19 +36841,19 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>24</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Mírně létané (50-100h)</t>
+          <t>Létané (100-200h)</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-03</t>
         </is>
       </c>
     </row>
@@ -39475,16 +36875,18 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Křídlo EN B UP KIBO X M 90-115kg Křídlo EN B UP KIBO X M 90-115kg 60 000,00 CZK EN B Velikost: M Vzletová hmotnost: 90 -</t>
+          <t>Křídlo EN B AXIS Pluto 3 ML 90-115kg Listovaný Žádné SIV Nevětveno Drobné opravy TK platná Křídlo EN B AXIS Pluto 3 ML 9</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/up-kibo-x-m-90-115kg-7824/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/axis-pluto-3-ml-90-115kg-concertinas-no-sivs-no-trees-sm-7858/</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
+      <c r="G3" t="n">
+        <v>2021</v>
+      </c>
       <c r="H3" t="inlineStr">
         <is>
           <t>EN B</t>
@@ -39492,19 +36894,19 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Jako nové (0-50h)</t>
+          <t>Mírně létané (50-100h)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-03</t>
         </is>
       </c>
     </row>
@@ -39526,38 +36928,34 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Křídlo EN B AXIS Pluto 2 M 80-105kg Křídlo EN B AXIS Pluto 2 M 80-105kg 4 000,00 CZK EN B Velikost: M Vzletová hmotnost:</t>
+          <t>Křídlo EN B Nova Mentor 4 80-105kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B Nova Mentor 4 8</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/axis-pluto-2-m-80-105kg-7822/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-4-80-105kg-no-sivs-no-flying-on-the-sand-no--7854/</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="n">
-        <v>2014</v>
+        <v>2018</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
           <t>EN B</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
+      <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Více létané (200-300h)</t>
+          <t>Jako nové (0-50h)</t>
         </is>
       </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-03</t>
         </is>
       </c>
     </row>
@@ -39579,17 +36977,17 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Křídlo EN B Ozone Rush 5 L 85-105kg Listovaný Nelétáno na písku Nekoupáno Drobné opravy TK platná Křídlo EN B Ozone Rush</t>
+          <t>Křídlo EN B SKY Paragliders Kudos 2 L 85-108kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá Křídlo EN B SK</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/ozone-rush-5-l-85-105kg-concertinas-no-flying-on-the-san-7815/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/sky-paragliders-kudos-2-l-85-108kg-no-sivs-no-flying-on--7852/</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="n">
-        <v>2019</v>
+        <v>2024</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -39604,13 +37002,13 @@
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Létané (100-200h)</t>
+          <t>Jako nové (0-50h)</t>
         </is>
       </c>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-03</t>
         </is>
       </c>
     </row>
@@ -39632,17 +37030,15 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Křídlo EN B AXIS Comet 3 M Listovaný Nové Žádné SIV Křídlo EN B AXIS Comet 3 M Listovaný Nové Žádné SIV 21 865,36 CZK (9</t>
+          <t>Křídlo EN B SKY Paragliders Kudos 2 M 74-94kg Listovaný Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B SKY</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-concertinas-new-no-sivs-7529/</t>
-        </is>
-      </c>
-      <c r="F6" t="n">
-        <v>900</v>
-      </c>
+          <t>https://paragliding-bazar.cz/cs/offering/sky-paragliders-kudos-2-m-74-94kg-concertinas-no-flying--7844/</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
       <c r="G6" t="n">
         <v>2020</v>
       </c>
@@ -39659,25 +37055,25 @@
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Jako nové (0-50h)</t>
+          <t>Mírně létané (50-100h)</t>
         </is>
       </c>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-03</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_a</t>
+          <t>paragliding_bazar_cz_b</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN A</t>
+          <t>Paragliding Bazar CZ – EN B</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -39687,38 +37083,40 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Křídlo EN A UP Dena M 85-110kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá TK platná Křídlo EN A UP Dena</t>
+          <t>Křídlo EN B Advance Epsilon DLS 26 Křídlo EN B Advance Epsilon DLS 26 41 394,76 CZK (1 700,00 EUR) EN B Velikost: 26 Opo</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/up-dena-m-85-110kg-no-sivs-no-flying-on-the-sand-no-tree-7839/</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr"/>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-dls-26-7734/</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>1700</v>
+      </c>
       <c r="G7" t="n">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>EN A</t>
+          <t>EN B</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>26</t>
         </is>
       </c>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Jako nové (0-50h)</t>
+          <t>Létané (100-200h)</t>
         </is>
       </c>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-03</t>
         </is>
       </c>
     </row>
@@ -39740,173 +37138,36 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Křídlo EN A GIN Bolero 5 m 85-105kg Drobné opravy TK platná Křídlo EN A GIN Bolero 5 m 85-105kg Drobné opravy TK platná</t>
+          <t>Křídlo EN A mac para Lucky 25 70-90kg Nelétáno na písku Nevětveno Nekoupáno Drobné opravy TK čerstvá Křídlo EN A mac par</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/gin-bolero-5-m-85-105kg-small-repairs-tc-valid-7814/</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr"/>
+          <t>https://paragliding-bazar.cz/cs/offering/mac-para-lucky-25-70-90kg-no-flying-on-the-sand-no-trees-7848/</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>390</v>
+      </c>
       <c r="G8" t="n">
-        <v>2015</v>
+        <v>2005</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
           <t>EN A</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>m</t>
-        </is>
-      </c>
+      <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Olétané (více než 300h)</t>
+          <t>Více létané (200-300h)</t>
         </is>
       </c>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>hochries_de</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>ADVANCE Sigma DLS 20</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>https://shop.flugschule-hochries.de/ADVANCE-Sigma-DLS-20/SW10843</t>
-        </is>
-      </c>
-      <c r="F9" t="n">
-        <v>3875</v>
-      </c>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>2026-09-26</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>hochries_de</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>ADVANCE Theta ULS 21</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>https://shop.flugschule-hochries.de/ADVANCE-Theta-ULS-21</t>
-        </is>
-      </c>
-      <c r="F10" t="n">
-        <v>3275</v>
-      </c>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>21</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>2026-09-26</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>hochries_de</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>ADVANCE Xi 23</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>https://shop.flugschule-hochries.de/ADVANCE-Xi-23</t>
-        </is>
-      </c>
-      <c r="F11" t="n">
-        <v>975</v>
-      </c>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>23</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>2026-09-26</t>
+          <t>2026-10-03</t>
         </is>
       </c>
     </row>
@@ -39921,255 +37182,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M4"/>
+  <dimension ref="A1:M1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="9" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="7" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="13" customWidth="1" min="13" max="13"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>source_id</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>source_name</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>country</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>url</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>price_eur</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>year</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>category</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>size</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>weight_range</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>condition</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>date_listed</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>date_found</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>paragliding_bazar_cz_b</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Paragliding Bazar CZ – EN B</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>CZ</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Křídlo EN B AXIS Comet 3 M Listovaný Nové Žádné SIV Křídlo EN B AXIS Comet 3 M Listovaný Nové Žádné SIV 21 865,36 CZK (9</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>https://paragliding-bazar.cz/cs/offering/axis-comet-3-m-concertinas-new-no-sivs-7529/</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>900</v>
-      </c>
-      <c r="G2" t="n">
-        <v>2020</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>EN B</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Jako nové (0-50h)</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>2026-09-26</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>hochries_de</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>ADVANCE Theta ULS 21</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>https://shop.flugschule-hochries.de/ADVANCE-Theta-ULS-21</t>
-        </is>
-      </c>
-      <c r="F3" t="n">
-        <v>3275</v>
-      </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>21</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>2026-09-26</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>hochries_de</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>ADVANCE Xi 23</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>https://shop.flugschule-hochries.de/ADVANCE-Xi-23</t>
-        </is>
-      </c>
-      <c r="F4" t="n">
-        <v>975</v>
-      </c>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>23</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>2026-09-26</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:M2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="42" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="52" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="6" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="7" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
@@ -40247,48 +37267,99 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>hochries_de</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>ADVANCE Xi 23</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>https://shop.flugschule-hochries.de/ADVANCE-Xi-23</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>975</v>
-      </c>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>23</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>2026-09-26</t>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="6" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>source_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>source_name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>url</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>price_eur</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>year</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>size</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>weight_range</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>condition</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>date_listed</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>date_found</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: bazar_watcher data update 2026-10-10
</commit_message>
<xml_diff>
--- a/data/bazar_watcher/listings.xlsx
+++ b/data/bazar_watcher/listings.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M656"/>
+  <dimension ref="A1:M676"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -35905,8 +35905,10 @@
         </is>
       </c>
       <c r="F650" t="inlineStr"/>
-      <c r="G650" t="n">
-        <v>2019</v>
+      <c r="G650" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
       </c>
       <c r="H650" t="inlineStr">
         <is>
@@ -35958,8 +35960,10 @@
         </is>
       </c>
       <c r="F651" t="inlineStr"/>
-      <c r="G651" t="n">
-        <v>2021</v>
+      <c r="G651" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
       </c>
       <c r="H651" t="inlineStr">
         <is>
@@ -36011,8 +36015,10 @@
         </is>
       </c>
       <c r="F652" t="inlineStr"/>
-      <c r="G652" t="n">
-        <v>2018</v>
+      <c r="G652" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
       </c>
       <c r="H652" t="inlineStr">
         <is>
@@ -36060,8 +36066,10 @@
         </is>
       </c>
       <c r="F653" t="inlineStr"/>
-      <c r="G653" t="n">
-        <v>2024</v>
+      <c r="G653" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
       </c>
       <c r="H653" t="inlineStr">
         <is>
@@ -36113,8 +36121,10 @@
         </is>
       </c>
       <c r="F654" t="inlineStr"/>
-      <c r="G654" t="n">
-        <v>2020</v>
+      <c r="G654" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
       </c>
       <c r="H654" t="inlineStr">
         <is>
@@ -36165,11 +36175,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-dls-26-7734/</t>
         </is>
       </c>
-      <c r="F655" t="n">
-        <v>1700</v>
-      </c>
-      <c r="G655" t="n">
-        <v>2023</v>
+      <c r="F655" t="inlineStr">
+        <is>
+          <t>1700.0</t>
+        </is>
+      </c>
+      <c r="G655" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
       </c>
       <c r="H655" t="inlineStr">
         <is>
@@ -36220,11 +36234,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/mac-para-lucky-25-70-90kg-no-flying-on-the-sand-no-trees-7848/</t>
         </is>
       </c>
-      <c r="F656" t="n">
-        <v>390</v>
-      </c>
-      <c r="G656" t="n">
-        <v>2005</v>
+      <c r="F656" t="inlineStr">
+        <is>
+          <t>390.0</t>
+        </is>
+      </c>
+      <c r="G656" t="inlineStr">
+        <is>
+          <t>2005</t>
+        </is>
       </c>
       <c r="H656" t="inlineStr">
         <is>
@@ -36242,6 +36260,1026 @@
       <c r="M656" t="inlineStr">
         <is>
           <t>2026-10-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="657">
+      <c r="A657" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B657" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C657" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D657" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Advance Epsilon DLS 26 Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B Advan</t>
+        </is>
+      </c>
+      <c r="E657" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-dls-26-concertinas-no-sivs-no-flying-on--7898/</t>
+        </is>
+      </c>
+      <c r="F657" t="inlineStr"/>
+      <c r="G657" t="n">
+        <v>2025</v>
+      </c>
+      <c r="H657" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I657" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="J657" t="inlineStr"/>
+      <c r="K657" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L657" t="inlineStr"/>
+      <c r="M657" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="658">
+      <c r="A658" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B658" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C658" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D658" t="inlineStr">
+        <is>
+          <t>Křídlo EN B SKY Paragliders Kudos 2 M 74-94kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá Křídlo EN B SKY</t>
+        </is>
+      </c>
+      <c r="E658" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/sky-paragliders-kudos-2-m-74-94kg-no-sivs-no-flying-on-t-7892/</t>
+        </is>
+      </c>
+      <c r="F658" t="inlineStr"/>
+      <c r="G658" t="n">
+        <v>2024</v>
+      </c>
+      <c r="H658" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I658" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J658" t="inlineStr"/>
+      <c r="K658" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L658" t="inlineStr"/>
+      <c r="M658" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="659">
+      <c r="A659" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B659" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C659" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D659" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AirDesign soar M 85-105kg Listovaný Odlehčeno Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Křídlo EN B Ai</t>
+        </is>
+      </c>
+      <c r="E659" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/airdesign-soar-m-85-105kg-concertinas-lightened-no-sivs--7889/</t>
+        </is>
+      </c>
+      <c r="F659" t="inlineStr"/>
+      <c r="G659" t="n">
+        <v>2022</v>
+      </c>
+      <c r="H659" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I659" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J659" t="inlineStr"/>
+      <c r="K659" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L659" t="inlineStr"/>
+      <c r="M659" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="660">
+      <c r="A660" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B660" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C660" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D660" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Nova Mentor 6 L 100-130kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Křídlo EN B Nova Mentor 6 L 100-13</t>
+        </is>
+      </c>
+      <c r="E660" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-6-l-100-130kg-no-sivs-no-flying-on-the-sand--7879/</t>
+        </is>
+      </c>
+      <c r="F660" t="n">
+        <v>800</v>
+      </c>
+      <c r="G660" t="n">
+        <v>2019</v>
+      </c>
+      <c r="H660" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I660" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J660" t="inlineStr"/>
+      <c r="K660" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L660" t="inlineStr"/>
+      <c r="M660" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="661">
+      <c r="A661" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B661" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C661" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D661" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Drift Hawk L 95-119kg Listovaný Nelétáno na písku Nekoupáno Drobné opravy TK čerstvá TK platná Křídlo EN B D</t>
+        </is>
+      </c>
+      <c r="E661" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/drift-hawk-l-95-119kg-concertinas-no-flying-on-the-sand--7870/</t>
+        </is>
+      </c>
+      <c r="F661" t="n">
+        <v>1739</v>
+      </c>
+      <c r="G661" t="n">
+        <v>2024</v>
+      </c>
+      <c r="H661" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I661" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J661" t="inlineStr"/>
+      <c r="K661" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L661" t="inlineStr"/>
+      <c r="M661" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="662">
+      <c r="A662" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B662" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C662" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D662" t="inlineStr">
+        <is>
+          <t>Křídlo EN B UP Kibo 2 M 85-110kg Křídlo EN B UP Kibo 2 M 85-110kg 33 000,00 CZK EN B Velikost: M Vzletová hmotnost: 85 -</t>
+        </is>
+      </c>
+      <c r="E662" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/up-kibo-2-m-85-110kg-7866/</t>
+        </is>
+      </c>
+      <c r="F662" t="inlineStr"/>
+      <c r="G662" t="n">
+        <v>2022</v>
+      </c>
+      <c r="H662" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I662" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J662" t="inlineStr"/>
+      <c r="K662" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L662" t="inlineStr"/>
+      <c r="M662" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="663">
+      <c r="A663" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B663" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C663" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D663" t="inlineStr">
+        <is>
+          <t>Křídlo EN B UP Summit XC 4 M 90-115kg Listovaný TK platná Křídlo EN B UP Summit XC 4 M 90-115kg Listovaný TK platná Nabí</t>
+        </is>
+      </c>
+      <c r="E663" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/up-summit-xc-4-m-90-115kg-concertinas-tc-valid-7828/</t>
+        </is>
+      </c>
+      <c r="F663" t="inlineStr"/>
+      <c r="G663" t="n">
+        <v>2021</v>
+      </c>
+      <c r="H663" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I663" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J663" t="inlineStr"/>
+      <c r="K663" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L663" t="inlineStr"/>
+      <c r="M663" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="664">
+      <c r="A664" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B664" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C664" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D664" t="inlineStr">
+        <is>
+          <t>Křídlo EN B UP KIBO X M 90-115kg Křídlo EN B UP KIBO X M 90-115kg 55 000,00 CZK EN B Velikost: M Vzletová hmotnost: 90 -</t>
+        </is>
+      </c>
+      <c r="E664" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/up-kibo-x-m-90-115kg-7824/</t>
+        </is>
+      </c>
+      <c r="F664" t="inlineStr"/>
+      <c r="G664" t="inlineStr"/>
+      <c r="H664" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I664" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J664" t="inlineStr"/>
+      <c r="K664" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L664" t="inlineStr"/>
+      <c r="M664" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="665">
+      <c r="A665" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B665" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C665" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D665" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Advance Epsilon DLS 26 Křídlo EN B Advance Epsilon DLS 26 41 301,23 CZK (1 700,00 EUR) EN B Velikost: 26 Opo</t>
+        </is>
+      </c>
+      <c r="E665" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-dls-26-7734/</t>
+        </is>
+      </c>
+      <c r="F665" t="n">
+        <v>1700</v>
+      </c>
+      <c r="G665" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H665" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I665" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="J665" t="inlineStr"/>
+      <c r="K665" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L665" t="inlineStr"/>
+      <c r="M665" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="666">
+      <c r="A666" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B666" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C666" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D666" t="inlineStr">
+        <is>
+          <t>Křídlo EN A UP Dena S 65-85kg Listovaný Nelétáno na písku Nevětveno Nekoupáno TK platná S batohem Křídlo EN A UP Dena S</t>
+        </is>
+      </c>
+      <c r="E666" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/up-dena-s-65-85kg-concertinas-no-flying-on-the-sand-no-t-7871/</t>
+        </is>
+      </c>
+      <c r="F666" t="inlineStr"/>
+      <c r="G666" t="n">
+        <v>2021</v>
+      </c>
+      <c r="H666" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I666" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J666" t="inlineStr"/>
+      <c r="K666" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L666" t="inlineStr"/>
+      <c r="M666" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="667">
+      <c r="A667" t="inlineStr">
+        <is>
+          <t>paragliding_store_at</t>
+        </is>
+      </c>
+      <c r="B667" t="inlineStr">
+        <is>
+          <t>Paragliding Store AT – Used</t>
+        </is>
+      </c>
+      <c r="C667" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="D667" t="inlineStr">
+        <is>
+          <t>Advance Epsilon 10 DLS 26</t>
+        </is>
+      </c>
+      <c r="E667" t="inlineStr">
+        <is>
+          <t>https://www.paragliding-store.at/shop/gebrauchtmarkt-used-stuff/used-paragliders/</t>
+        </is>
+      </c>
+      <c r="F667" t="n">
+        <v>2690</v>
+      </c>
+      <c r="G667" t="n">
+        <v>2024</v>
+      </c>
+      <c r="H667" t="inlineStr"/>
+      <c r="I667" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="J667" t="inlineStr">
+        <is>
+          <t>79kg-103kg</t>
+        </is>
+      </c>
+      <c r="K667" t="inlineStr">
+        <is>
+          <t>sehr guter Zustand ca</t>
+        </is>
+      </c>
+      <c r="L667" t="inlineStr"/>
+      <c r="M667" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="668">
+      <c r="A668" t="inlineStr">
+        <is>
+          <t>paragliding_store_at</t>
+        </is>
+      </c>
+      <c r="B668" t="inlineStr">
+        <is>
+          <t>Paragliding Store AT – Used</t>
+        </is>
+      </c>
+      <c r="C668" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="D668" t="inlineStr">
+        <is>
+          <t>Advance Epsilon 10 DLS 24</t>
+        </is>
+      </c>
+      <c r="E668" t="inlineStr">
+        <is>
+          <t>https://www.paragliding-store.at/shop/gebrauchtmarkt-used-stuff/used-paragliders/</t>
+        </is>
+      </c>
+      <c r="F668" t="n">
+        <v>2940</v>
+      </c>
+      <c r="G668" t="n">
+        <v>2025</v>
+      </c>
+      <c r="H668" t="inlineStr"/>
+      <c r="I668" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="J668" t="inlineStr">
+        <is>
+          <t>67kg-90kg</t>
+        </is>
+      </c>
+      <c r="K668" t="inlineStr">
+        <is>
+          <t>sehr guter Zustand ca</t>
+        </is>
+      </c>
+      <c r="L668" t="inlineStr"/>
+      <c r="M668" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="669">
+      <c r="A669" t="inlineStr">
+        <is>
+          <t>paragliding_store_at</t>
+        </is>
+      </c>
+      <c r="B669" t="inlineStr">
+        <is>
+          <t>Paragliding Store AT – Used</t>
+        </is>
+      </c>
+      <c r="C669" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="D669" t="inlineStr">
+        <is>
+          <t>Advance Epsilon 10 DLS 28</t>
+        </is>
+      </c>
+      <c r="E669" t="inlineStr">
+        <is>
+          <t>https://www.paragliding-store.at/shop/gebrauchtmarkt-used-stuff/used-paragliders/</t>
+        </is>
+      </c>
+      <c r="F669" t="n">
+        <v>2940</v>
+      </c>
+      <c r="G669" t="n">
+        <v>2025</v>
+      </c>
+      <c r="H669" t="inlineStr"/>
+      <c r="I669" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J669" t="inlineStr">
+        <is>
+          <t>91kg-118kg</t>
+        </is>
+      </c>
+      <c r="K669" t="inlineStr">
+        <is>
+          <t>sehr sehr guter Zustand ca</t>
+        </is>
+      </c>
+      <c r="L669" t="inlineStr"/>
+      <c r="M669" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="670">
+      <c r="A670" t="inlineStr">
+        <is>
+          <t>paragliding_store_at</t>
+        </is>
+      </c>
+      <c r="B670" t="inlineStr">
+        <is>
+          <t>Paragliding Store AT – Used</t>
+        </is>
+      </c>
+      <c r="C670" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="D670" t="inlineStr">
+        <is>
+          <t>Advance Theta 27</t>
+        </is>
+      </c>
+      <c r="E670" t="inlineStr">
+        <is>
+          <t>https://www.paragliding-store.at/shop/gebrauchtmarkt-used-stuff/used-paragliders/</t>
+        </is>
+      </c>
+      <c r="F670" t="n">
+        <v>2640</v>
+      </c>
+      <c r="G670" t="n">
+        <v>2024</v>
+      </c>
+      <c r="H670" t="inlineStr"/>
+      <c r="I670" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="J670" t="inlineStr">
+        <is>
+          <t>90kg-112kg</t>
+        </is>
+      </c>
+      <c r="K670" t="inlineStr">
+        <is>
+          <t>sehr guter Zustand, keine Beschädigungen</t>
+        </is>
+      </c>
+      <c r="L670" t="inlineStr"/>
+      <c r="M670" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="671">
+      <c r="A671" t="inlineStr">
+        <is>
+          <t>paragliding_store_at</t>
+        </is>
+      </c>
+      <c r="B671" t="inlineStr">
+        <is>
+          <t>Paragliding Store AT – Used</t>
+        </is>
+      </c>
+      <c r="C671" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="D671" t="inlineStr">
+        <is>
+          <t>Advance Theta 25</t>
+        </is>
+      </c>
+      <c r="E671" t="inlineStr">
+        <is>
+          <t>https://www.paragliding-store.at/shop/gebrauchtmarkt-used-stuff/used-paragliders/</t>
+        </is>
+      </c>
+      <c r="F671" t="n">
+        <v>3890</v>
+      </c>
+      <c r="G671" t="n">
+        <v>2026</v>
+      </c>
+      <c r="H671" t="inlineStr"/>
+      <c r="I671" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="J671" t="inlineStr">
+        <is>
+          <t>79kg-99kg</t>
+        </is>
+      </c>
+      <c r="K671" t="inlineStr">
+        <is>
+          <t>sehr sehr guter Zustand, keine Beschädig</t>
+        </is>
+      </c>
+      <c r="L671" t="inlineStr"/>
+      <c r="M671" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="672">
+      <c r="A672" t="inlineStr">
+        <is>
+          <t>parafly_at</t>
+        </is>
+      </c>
+      <c r="B672" t="inlineStr">
+        <is>
+          <t>Parafly AT – Gebrauchtmarkt</t>
+        </is>
+      </c>
+      <c r="C672" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="D672" t="inlineStr">
+        <is>
+          <t>Advance PI ULS 14m²</t>
+        </is>
+      </c>
+      <c r="E672" t="inlineStr">
+        <is>
+          <t>https://shop.parafly.at/produkt/advance-pi-uls-14m%c2%b2/</t>
+        </is>
+      </c>
+      <c r="F672" t="n">
+        <v>2600</v>
+      </c>
+      <c r="G672" t="inlineStr"/>
+      <c r="H672" t="inlineStr"/>
+      <c r="I672" t="inlineStr"/>
+      <c r="J672" t="inlineStr"/>
+      <c r="K672" t="inlineStr"/>
+      <c r="L672" t="inlineStr"/>
+      <c r="M672" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="673">
+      <c r="A673" t="inlineStr">
+        <is>
+          <t>parafly_at</t>
+        </is>
+      </c>
+      <c r="B673" t="inlineStr">
+        <is>
+          <t>Parafly AT – Gebrauchtmarkt</t>
+        </is>
+      </c>
+      <c r="C673" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="D673" t="inlineStr">
+        <is>
+          <t>Gleitschirm Komplettset Hike&amp;Fly</t>
+        </is>
+      </c>
+      <c r="E673" t="inlineStr">
+        <is>
+          <t>https://shop.parafly.at/produkt/gleitschirm-komplettset-hikefly/</t>
+        </is>
+      </c>
+      <c r="F673" t="n">
+        <v>3800</v>
+      </c>
+      <c r="G673" t="inlineStr"/>
+      <c r="H673" t="inlineStr"/>
+      <c r="I673" t="inlineStr"/>
+      <c r="J673" t="inlineStr"/>
+      <c r="K673" t="inlineStr"/>
+      <c r="L673" t="inlineStr"/>
+      <c r="M673" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="674">
+      <c r="A674" t="inlineStr">
+        <is>
+          <t>parafly_at</t>
+        </is>
+      </c>
+      <c r="B674" t="inlineStr">
+        <is>
+          <t>Parafly AT – Gebrauchtmarkt</t>
+        </is>
+      </c>
+      <c r="C674" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="D674" t="inlineStr">
+        <is>
+          <t>Gin Explorer 2</t>
+        </is>
+      </c>
+      <c r="E674" t="inlineStr">
+        <is>
+          <t>https://shop.parafly.at/produkt/gin-explorer-2/</t>
+        </is>
+      </c>
+      <c r="F674" t="n">
+        <v>2300</v>
+      </c>
+      <c r="G674" t="inlineStr"/>
+      <c r="H674" t="inlineStr"/>
+      <c r="I674" t="inlineStr"/>
+      <c r="J674" t="inlineStr"/>
+      <c r="K674" t="inlineStr"/>
+      <c r="L674" t="inlineStr"/>
+      <c r="M674" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="675">
+      <c r="A675" t="inlineStr">
+        <is>
+          <t>hochries_de</t>
+        </is>
+      </c>
+      <c r="B675" t="inlineStr">
+        <is>
+          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
+        </is>
+      </c>
+      <c r="C675" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D675" t="inlineStr">
+        <is>
+          <t>ADVANCE Lightness 3 M - S</t>
+        </is>
+      </c>
+      <c r="E675" t="inlineStr">
+        <is>
+          <t>https://shop.flugschule-hochries.de/ADVANCE-Lightness-3-M-S/SW10950</t>
+        </is>
+      </c>
+      <c r="F675" t="n">
+        <v>745</v>
+      </c>
+      <c r="G675" t="inlineStr"/>
+      <c r="H675" t="inlineStr"/>
+      <c r="I675" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J675" t="inlineStr"/>
+      <c r="K675" t="inlineStr"/>
+      <c r="L675" t="inlineStr"/>
+      <c r="M675" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="676">
+      <c r="A676" t="inlineStr">
+        <is>
+          <t>paraglidingshop_ch</t>
+        </is>
+      </c>
+      <c r="B676" t="inlineStr">
+        <is>
+          <t>Paraglidingshop CH – Occasionen</t>
+        </is>
+      </c>
+      <c r="C676" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="D676" t="inlineStr">
+        <is>
+          <t>Companion SQR Light 190 Occassion</t>
+        </is>
+      </c>
+      <c r="E676" t="inlineStr">
+        <is>
+          <t>https://paraglidingshop.ch/Companion-SQR-Light-190-Occassion/SW10852</t>
+        </is>
+      </c>
+      <c r="F676" t="n">
+        <v>619</v>
+      </c>
+      <c r="G676" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H676" t="inlineStr"/>
+      <c r="I676" t="inlineStr"/>
+      <c r="J676" t="inlineStr"/>
+      <c r="K676" t="inlineStr"/>
+      <c r="L676" t="inlineStr"/>
+      <c r="M676" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
         </is>
       </c>
     </row>
@@ -36256,20 +37294,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M8"/>
+  <dimension ref="A1:M28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="25" customWidth="1" min="11" max="11"/>
+    <col width="43" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
@@ -36368,8 +37406,10 @@
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
-      <c r="G2" t="n">
-        <v>2019</v>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -36421,8 +37461,10 @@
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
-      <c r="G3" t="n">
-        <v>2021</v>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -36474,8 +37516,10 @@
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
-      <c r="G4" t="n">
-        <v>2018</v>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -36523,8 +37567,10 @@
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
-      <c r="G5" t="n">
-        <v>2024</v>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -36576,8 +37622,10 @@
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
-      <c r="G6" t="n">
-        <v>2020</v>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
@@ -36628,11 +37676,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-dls-26-7734/</t>
         </is>
       </c>
-      <c r="F7" t="n">
-        <v>1700</v>
-      </c>
-      <c r="G7" t="n">
-        <v>2023</v>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>1700.0</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -36683,11 +37735,15 @@
           <t>https://paragliding-bazar.cz/cs/offering/mac-para-lucky-25-70-90kg-no-flying-on-the-sand-no-trees-7848/</t>
         </is>
       </c>
-      <c r="F8" t="n">
-        <v>390</v>
-      </c>
-      <c r="G8" t="n">
-        <v>2005</v>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>390.0</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>2005</t>
+        </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
@@ -36705,6 +37761,1026 @@
       <c r="M8" t="inlineStr">
         <is>
           <t>2026-10-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Advance Epsilon DLS 26 Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B Advan</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-dls-26-concertinas-no-sivs-no-flying-on--7898/</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="n">
+        <v>2025</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Křídlo EN B SKY Paragliders Kudos 2 M 74-94kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá Křídlo EN B SKY</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/sky-paragliders-kudos-2-m-74-94kg-no-sivs-no-flying-on-t-7892/</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="n">
+        <v>2024</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Křídlo EN B AirDesign soar M 85-105kg Listovaný Odlehčeno Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Křídlo EN B Ai</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/airdesign-soar-m-85-105kg-concertinas-lightened-no-sivs--7889/</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="n">
+        <v>2022</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Nova Mentor 6 L 100-130kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Křídlo EN B Nova Mentor 6 L 100-13</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-6-l-100-130kg-no-sivs-no-flying-on-the-sand--7879/</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>800</v>
+      </c>
+      <c r="G12" t="n">
+        <v>2019</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Drift Hawk L 95-119kg Listovaný Nelétáno na písku Nekoupáno Drobné opravy TK čerstvá TK platná Křídlo EN B D</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/drift-hawk-l-95-119kg-concertinas-no-flying-on-the-sand--7870/</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>1739</v>
+      </c>
+      <c r="G13" t="n">
+        <v>2024</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Křídlo EN B UP Kibo 2 M 85-110kg Křídlo EN B UP Kibo 2 M 85-110kg 33 000,00 CZK EN B Velikost: M Vzletová hmotnost: 85 -</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/up-kibo-2-m-85-110kg-7866/</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="n">
+        <v>2022</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Křídlo EN B UP Summit XC 4 M 90-115kg Listovaný TK platná Křídlo EN B UP Summit XC 4 M 90-115kg Listovaný TK platná Nabí</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/up-summit-xc-4-m-90-115kg-concertinas-tc-valid-7828/</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="n">
+        <v>2021</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Křídlo EN B UP KIBO X M 90-115kg Křídlo EN B UP KIBO X M 90-115kg 55 000,00 CZK EN B Velikost: M Vzletová hmotnost: 90 -</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/up-kibo-x-m-90-115kg-7824/</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Advance Epsilon DLS 26 Křídlo EN B Advance Epsilon DLS 26 41 301,23 CZK (1 700,00 EUR) EN B Velikost: 26 Opo</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-dls-26-7734/</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>1700</v>
+      </c>
+      <c r="G17" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Křídlo EN A UP Dena S 65-85kg Listovaný Nelétáno na písku Nevětveno Nekoupáno TK platná S batohem Křídlo EN A UP Dena S</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/up-dena-s-65-85kg-concertinas-no-flying-on-the-sand-no-t-7871/</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="n">
+        <v>2021</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>paragliding_store_at</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Paragliding Store AT – Used</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Advance Epsilon 10 DLS 26</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>https://www.paragliding-store.at/shop/gebrauchtmarkt-used-stuff/used-paragliders/</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>2690</v>
+      </c>
+      <c r="G19" t="n">
+        <v>2024</v>
+      </c>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>79kg-103kg</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>sehr guter Zustand ca</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>paragliding_store_at</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Paragliding Store AT – Used</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Advance Epsilon 10 DLS 24</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>https://www.paragliding-store.at/shop/gebrauchtmarkt-used-stuff/used-paragliders/</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>2940</v>
+      </c>
+      <c r="G20" t="n">
+        <v>2025</v>
+      </c>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>67kg-90kg</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>sehr guter Zustand ca</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>paragliding_store_at</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Paragliding Store AT – Used</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Advance Epsilon 10 DLS 28</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>https://www.paragliding-store.at/shop/gebrauchtmarkt-used-stuff/used-paragliders/</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
+        <v>2940</v>
+      </c>
+      <c r="G21" t="n">
+        <v>2025</v>
+      </c>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>91kg-118kg</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>sehr sehr guter Zustand ca</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>paragliding_store_at</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Paragliding Store AT – Used</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Advance Theta 27</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>https://www.paragliding-store.at/shop/gebrauchtmarkt-used-stuff/used-paragliders/</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>2640</v>
+      </c>
+      <c r="G22" t="n">
+        <v>2024</v>
+      </c>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>90kg-112kg</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>sehr guter Zustand, keine Beschädigungen</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr"/>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>paragliding_store_at</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Paragliding Store AT – Used</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Advance Theta 25</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>https://www.paragliding-store.at/shop/gebrauchtmarkt-used-stuff/used-paragliders/</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>3890</v>
+      </c>
+      <c r="G23" t="n">
+        <v>2026</v>
+      </c>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>79kg-99kg</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>sehr sehr guter Zustand, keine Beschädig</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr"/>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>parafly_at</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Parafly AT – Gebrauchtmarkt</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Advance PI ULS 14m²</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>https://shop.parafly.at/produkt/advance-pi-uls-14m%c2%b2/</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>2600</v>
+      </c>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" t="inlineStr"/>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>parafly_at</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Parafly AT – Gebrauchtmarkt</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Gleitschirm Komplettset Hike&amp;Fly</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>https://shop.parafly.at/produkt/gleitschirm-komplettset-hikefly/</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
+        <v>3800</v>
+      </c>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr"/>
+      <c r="K25" t="inlineStr"/>
+      <c r="L25" t="inlineStr"/>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>parafly_at</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Parafly AT – Gebrauchtmarkt</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Gin Explorer 2</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>https://shop.parafly.at/produkt/gin-explorer-2/</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>2300</v>
+      </c>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" t="inlineStr"/>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>hochries_de</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>ADVANCE Lightness 3 M - S</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>https://shop.flugschule-hochries.de/ADVANCE-Lightness-3-M-S/SW10950</t>
+        </is>
+      </c>
+      <c r="F27" t="n">
+        <v>745</v>
+      </c>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>paraglidingshop_ch</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Paraglidingshop CH – Occasionen</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Companion SQR Light 190 Occassion</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>https://paraglidingshop.ch/Companion-SQR-Light-190-Occassion/SW10852</t>
+        </is>
+      </c>
+      <c r="F28" t="n">
+        <v>619</v>
+      </c>
+      <c r="G28" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="inlineStr"/>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
         </is>
       </c>
     </row>
@@ -36719,20 +38795,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M8"/>
+  <dimension ref="A1:M21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="25" customWidth="1" min="11" max="11"/>
+    <col width="43" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
@@ -36822,17 +38898,17 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Křídlo EN B MAC Illusion 24 70-90kg Nelétáno na písku Nevětveno Nekoupáno TK čerstvá S listovacím obalem Křídlo EN B MAC</t>
+          <t>Křídlo EN B Advance Epsilon DLS 26 Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B Advan</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/mac-illusion-24-70-90kg-no-flying-on-the-sand-no-trees-n-7863/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-dls-26-concertinas-no-sivs-no-flying-on--7898/</t>
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="n">
-        <v>2019</v>
+        <v>2025</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -36841,19 +38917,19 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>26</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Létané (100-200h)</t>
+          <t>Mírně létané (50-100h)</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-10</t>
         </is>
       </c>
     </row>
@@ -36875,17 +38951,17 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Křídlo EN B AXIS Pluto 3 ML 90-115kg Listovaný Žádné SIV Nevětveno Drobné opravy TK platná Křídlo EN B AXIS Pluto 3 ML 9</t>
+          <t>Křídlo EN B SKY Paragliders Kudos 2 M 74-94kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá Křídlo EN B SKY</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/axis-pluto-3-ml-90-115kg-concertinas-no-sivs-no-trees-sm-7858/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/sky-paragliders-kudos-2-m-74-94kg-no-sivs-no-flying-on-t-7892/</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="n">
-        <v>2021</v>
+        <v>2024</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -36894,19 +38970,19 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>M</t>
         </is>
       </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Mírně létané (50-100h)</t>
+          <t>Jako nové (0-50h)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-10</t>
         </is>
       </c>
     </row>
@@ -36928,34 +39004,38 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Křídlo EN B Nova Mentor 4 80-105kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B Nova Mentor 4 8</t>
+          <t>Křídlo EN B AirDesign soar M 85-105kg Listovaný Odlehčeno Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Křídlo EN B Ai</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-4-80-105kg-no-sivs-no-flying-on-the-sand-no--7854/</t>
+          <t>https://paragliding-bazar.cz/cs/offering/airdesign-soar-m-85-105kg-concertinas-lightened-no-sivs--7889/</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="n">
-        <v>2018</v>
+        <v>2022</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
           <t>EN B</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Jako nové (0-50h)</t>
+          <t>Mírně létané (50-100h)</t>
         </is>
       </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-10</t>
         </is>
       </c>
     </row>
@@ -36977,17 +39057,19 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Křídlo EN B SKY Paragliders Kudos 2 L 85-108kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK čerstvá Křídlo EN B SK</t>
+          <t>Křídlo EN B Nova Mentor 6 L 100-130kg Žádné SIV Nelétáno na písku Nevětveno Nekoupáno Křídlo EN B Nova Mentor 6 L 100-13</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/sky-paragliders-kudos-2-l-85-108kg-no-sivs-no-flying-on--7852/</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr"/>
+          <t>https://paragliding-bazar.cz/cs/offering/nova-mentor-6-l-100-130kg-no-sivs-no-flying-on-the-sand--7879/</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>800</v>
+      </c>
       <c r="G5" t="n">
-        <v>2024</v>
+        <v>2019</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -37002,13 +39084,13 @@
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Jako nové (0-50h)</t>
+          <t>Létané (100-200h)</t>
         </is>
       </c>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-10</t>
         </is>
       </c>
     </row>
@@ -37030,17 +39112,19 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Křídlo EN B SKY Paragliders Kudos 2 M 74-94kg Listovaný Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B SKY</t>
+          <t>Křídlo EN B Drift Hawk L 95-119kg Listovaný Nelétáno na písku Nekoupáno Drobné opravy TK čerstvá TK platná Křídlo EN B D</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/sky-paragliders-kudos-2-m-74-94kg-concertinas-no-flying--7844/</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr"/>
+          <t>https://paragliding-bazar.cz/cs/offering/drift-hawk-l-95-119kg-concertinas-no-flying-on-the-sand--7870/</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>1739</v>
+      </c>
       <c r="G6" t="n">
-        <v>2020</v>
+        <v>2024</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
@@ -37049,7 +39133,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>L</t>
         </is>
       </c>
       <c r="J6" t="inlineStr"/>
@@ -37061,7 +39145,7 @@
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-10</t>
         </is>
       </c>
     </row>
@@ -37083,19 +39167,17 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Křídlo EN B Advance Epsilon DLS 26 Křídlo EN B Advance Epsilon DLS 26 41 394,76 CZK (1 700,00 EUR) EN B Velikost: 26 Opo</t>
+          <t>Křídlo EN B UP Kibo 2 M 85-110kg Křídlo EN B UP Kibo 2 M 85-110kg 33 000,00 CZK EN B Velikost: M Vzletová hmotnost: 85 -</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-dls-26-7734/</t>
-        </is>
-      </c>
-      <c r="F7" t="n">
-        <v>1700</v>
-      </c>
+          <t>https://paragliding-bazar.cz/cs/offering/up-kibo-2-m-85-110kg-7866/</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
       <c r="G7" t="n">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -37104,7 +39186,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>M</t>
         </is>
       </c>
       <c r="J7" t="inlineStr"/>
@@ -37116,19 +39198,19 @@
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-10</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>paragliding_bazar_cz_a</t>
+          <t>paragliding_bazar_cz_b</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Paragliding Bazar CZ – EN A</t>
+          <t>Paragliding Bazar CZ – EN B</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -37138,36 +39220,683 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Křídlo EN A mac para Lucky 25 70-90kg Nelétáno na písku Nevětveno Nekoupáno Drobné opravy TK čerstvá Křídlo EN A mac par</t>
+          <t>Křídlo EN B UP Summit XC 4 M 90-115kg Listovaný TK platná Křídlo EN B UP Summit XC 4 M 90-115kg Listovaný TK platná Nabí</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://paragliding-bazar.cz/cs/offering/mac-para-lucky-25-70-90kg-no-flying-on-the-sand-no-trees-7848/</t>
-        </is>
-      </c>
-      <c r="F8" t="n">
-        <v>390</v>
-      </c>
+          <t>https://paragliding-bazar.cz/cs/offering/up-summit-xc-4-m-90-115kg-concertinas-tc-valid-7828/</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr"/>
       <c r="G8" t="n">
-        <v>2005</v>
+        <v>2021</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>EN A</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr"/>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Více létané (200-300h)</t>
+          <t>Mírně létané (50-100h)</t>
         </is>
       </c>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Křídlo EN B UP KIBO X M 90-115kg Křídlo EN B UP KIBO X M 90-115kg 55 000,00 CZK EN B Velikost: M Vzletová hmotnost: 90 -</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/up-kibo-x-m-90-115kg-7824/</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Jako nové (0-50h)</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Advance Epsilon DLS 26 Křídlo EN B Advance Epsilon DLS 26 41 301,23 CZK (1 700,00 EUR) EN B Velikost: 26 Opo</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-dls-26-7734/</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>1700</v>
+      </c>
+      <c r="G10" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Křídlo EN A UP Dena S 65-85kg Listovaný Nelétáno na písku Nevětveno Nekoupáno TK platná S batohem Křídlo EN A UP Dena S</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/up-dena-s-65-85kg-concertinas-no-flying-on-the-sand-no-t-7871/</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="n">
+        <v>2021</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>paragliding_store_at</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Paragliding Store AT – Used</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Advance Epsilon 10 DLS 26</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>https://www.paragliding-store.at/shop/gebrauchtmarkt-used-stuff/used-paragliders/</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>2690</v>
+      </c>
+      <c r="G12" t="n">
+        <v>2024</v>
+      </c>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>79kg-103kg</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>sehr guter Zustand ca</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>paragliding_store_at</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Paragliding Store AT – Used</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Advance Epsilon 10 DLS 24</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>https://www.paragliding-store.at/shop/gebrauchtmarkt-used-stuff/used-paragliders/</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>2940</v>
+      </c>
+      <c r="G13" t="n">
+        <v>2025</v>
+      </c>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>67kg-90kg</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>sehr guter Zustand ca</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>paragliding_store_at</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Paragliding Store AT – Used</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Advance Epsilon 10 DLS 28</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>https://www.paragliding-store.at/shop/gebrauchtmarkt-used-stuff/used-paragliders/</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>2940</v>
+      </c>
+      <c r="G14" t="n">
+        <v>2025</v>
+      </c>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>91kg-118kg</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>sehr sehr guter Zustand ca</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>paragliding_store_at</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Paragliding Store AT – Used</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Advance Theta 27</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>https://www.paragliding-store.at/shop/gebrauchtmarkt-used-stuff/used-paragliders/</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>2640</v>
+      </c>
+      <c r="G15" t="n">
+        <v>2024</v>
+      </c>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>90kg-112kg</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>sehr guter Zustand, keine Beschädigungen</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>paragliding_store_at</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Paragliding Store AT – Used</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Advance Theta 25</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>https://www.paragliding-store.at/shop/gebrauchtmarkt-used-stuff/used-paragliders/</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>3890</v>
+      </c>
+      <c r="G16" t="n">
+        <v>2026</v>
+      </c>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>79kg-99kg</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>sehr sehr guter Zustand, keine Beschädig</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>parafly_at</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Parafly AT – Gebrauchtmarkt</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Advance PI ULS 14m²</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>https://shop.parafly.at/produkt/advance-pi-uls-14m%c2%b2/</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>2600</v>
+      </c>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>parafly_at</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Parafly AT – Gebrauchtmarkt</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Gleitschirm Komplettset Hike&amp;Fly</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>https://shop.parafly.at/produkt/gleitschirm-komplettset-hikefly/</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>3800</v>
+      </c>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>parafly_at</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Parafly AT – Gebrauchtmarkt</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Gin Explorer 2</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>https://shop.parafly.at/produkt/gin-explorer-2/</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>2300</v>
+      </c>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>hochries_de</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>ADVANCE Lightness 3 M - S</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>https://shop.flugschule-hochries.de/ADVANCE-Lightness-3-M-S/SW10950</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>745</v>
+      </c>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>paraglidingshop_ch</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Paraglidingshop CH – Occasionen</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Companion SQR Light 190 Occassion</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>https://paraglidingshop.ch/Companion-SQR-Light-190-Occassion/SW10852</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
+        <v>619</v>
+      </c>
+      <c r="G21" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
         </is>
       </c>
     </row>
@@ -37182,20 +39911,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:M5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="6" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="25" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
@@ -37264,6 +39993,214 @@
       <c r="M1" t="inlineStr">
         <is>
           <t>date_found</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Advance Epsilon DLS 26 Křídlo EN B Advance Epsilon DLS 26 41 301,23 CZK (1 700,00 EUR) EN B Velikost: 26 Opo</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-dls-26-7734/</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>1700</v>
+      </c>
+      <c r="G2" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Létané (100-200h)</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Křídlo EN A UP Dena S 65-85kg Listovaný Nelétáno na písku Nevětveno Nekoupáno TK platná S batohem Křídlo EN A UP Dena S</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/up-dena-s-65-85kg-concertinas-no-flying-on-the-sand-no-t-7871/</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="n">
+        <v>2021</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>paragliding_store_at</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Paragliding Store AT – Used</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Advance Epsilon 10 DLS 24</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>https://www.paragliding-store.at/shop/gebrauchtmarkt-used-stuff/used-paragliders/</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>2940</v>
+      </c>
+      <c r="G4" t="n">
+        <v>2025</v>
+      </c>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>67kg-90kg</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>sehr guter Zustand ca</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>hochries_de</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>ADVANCE Lightness 3 M - S</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>https://shop.flugschule-hochries.de/ADVANCE-Lightness-3-M-S/SW10950</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>745</v>
+      </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
         </is>
       </c>
     </row>
@@ -37278,20 +40215,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:M4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="6" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="25" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
@@ -37363,6 +40300,157 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_b</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN B</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Křídlo EN B Advance Epsilon DLS 26 Listovaný Žádné SIV Nelétáno na písku Nevětveno Nekoupáno TK platná Křídlo EN B Advan</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/advance-epsilon-dls-26-concertinas-no-sivs-no-flying-on--7898/</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="n">
+        <v>2025</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>EN B</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>paragliding_bazar_cz_a</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Paragliding Bazar CZ – EN A</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>CZ</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Křídlo EN A UP Dena S 65-85kg Listovaný Nelétáno na písku Nevětveno Nekoupáno TK platná S batohem Křídlo EN A UP Dena S</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>https://paragliding-bazar.cz/cs/offering/up-dena-s-65-85kg-concertinas-no-flying-on-the-sand-no-t-7871/</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="n">
+        <v>2021</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>EN A</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Mírně létané (50-100h)</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>hochries_de</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Flugschule Hochries DE – Gebrauchtmarkt</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>ADVANCE Lightness 3 M - S</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>https://shop.flugschule-hochries.de/ADVANCE-Lightness-3-M-S/SW10950</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>745</v>
+      </c>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>